<commit_message>
docs: alertas en DynamoDB, cuentas en Cognito y RDS solo para configuración
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015SVKuYduNdeGeu8Q4SMcKp
</commit_message>
<xml_diff>
--- a/docs/nota-2/Induplac_Roles_Equipo.xlsx
+++ b/docs/nota-2/Induplac_Roles_Equipo.xlsx
@@ -122,7 +122,7 @@
     <t xml:space="preserve">Cloud, backend y ciberseguridad</t>
   </si>
   <si>
-    <t xml:space="preserve">AWS en el Learner Lab: API Gateway, Lambda (Python), DynamoDB, RDS PostgreSQL (usuarios, permisos, umbrales y alertas) y S3 para publicar el dashboard; reglas de alerta; Cognito con MFA; IAM, TLS y cumplimiento de la Ley 19.628.</t>
+    <t xml:space="preserve">AWS en el Learner Lab: API Gateway, Lambda (Python), DynamoDB, RDS PostgreSQL (permisos, umbrales y catálogo) y S3 para publicar el dashboard; reglas de alerta; Cognito con MFA; IAM, TLS y cumplimiento de la Ley 19.628.</t>
   </si>
   <si>
     <t xml:space="preserve">backend/, infrastructure/</t>
@@ -266,7 +266,7 @@
     <t xml:space="preserve">Listo</t>
   </si>
   <si>
-    <t xml:space="preserve">Tablas en DynamoDB (intervalos)</t>
+    <t xml:space="preserve">Tablas en DynamoDB (intervalos y alertas)</t>
   </si>
   <si>
     <t xml:space="preserve">Reglas de alerta (+20 % kW, UV ≥ 8, agua y fugas)</t>
@@ -275,7 +275,7 @@
     <t xml:space="preserve">Dashboard publicado en S3</t>
   </si>
   <si>
-    <t xml:space="preserve">RDS PostgreSQL: usuarios, permisos, umbrales y alertas (se enciende para la demo)</t>
+    <t xml:space="preserve">RDS PostgreSQL: permisos, umbrales y catálogo (se enciende para la demo)</t>
   </si>
   <si>
     <t xml:space="preserve">Re-deploy de la Lambda con alertas del Edge</t>

</xml_diff>

<commit_message>
docs: documentación al día con el estado del 21/10 (MVP funcionando)
- CONTEXTO, README y GUIA-EQUIPO: alertas en DynamoDB, cuentas en Cognito,
  RDS solo configuración; Edge, Wokwi, backend y Cognito marcados como hechos
- ADR-01 y modo-offline: las alertas ya no van en RDS
- EN-CURSO, NOTA-2, roles-raci-gantt y Excel: estados de las tareas al día
- conclusiones: limitación de Cognito sin integrar y siguientes pasos

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015SVKuYduNdeGeu8Q4SMcKp
</commit_message>
<xml_diff>
--- a/docs/nota-2/Induplac_Roles_Equipo.xlsx
+++ b/docs/nota-2/Induplac_Roles_Equipo.xlsx
@@ -1709,8 +1709,10 @@
       <c r="C6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D6" s="4" t="s">
-        <v>49</v>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>Listo (PR #18)</t>
+        </is>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1723,8 +1725,10 @@
       <c r="C7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>49</v>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>Listo (PR #18)</t>
+        </is>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1737,8 +1741,10 @@
       <c r="C8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="4" t="s">
-        <v>49</v>
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>Listo (PR #16)</t>
+        </is>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1751,8 +1757,10 @@
       <c r="C9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>57</v>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1765,8 +1773,10 @@
       <c r="C10" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="4" t="s">
-        <v>49</v>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>Listo Local 1 (PR #16)</t>
+        </is>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1779,8 +1789,10 @@
       <c r="C11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D11" s="4" t="s">
-        <v>49</v>
+      <c r="D11" s="4" t="inlineStr">
+        <is>
+          <t>Listo (PR #16)</t>
+        </is>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1793,8 +1805,10 @@
       <c r="C12" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>49</v>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>Listo (PR #16)</t>
+        </is>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1807,8 +1821,10 @@
       <c r="C13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="4" t="s">
-        <v>57</v>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>Listo (PR #16)</t>
+        </is>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1821,8 +1837,10 @@
       <c r="C14" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>57</v>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>En curso</t>
+        </is>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1947,8 +1965,10 @@
       <c r="C23" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D23" s="4" t="s">
-        <v>49</v>
+      <c r="D23" s="4" t="inlineStr">
+        <is>
+          <t>Listo (PR #16)</t>
+        </is>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1961,8 +1981,10 @@
       <c r="C24" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D24" s="4" t="s">
-        <v>57</v>
+      <c r="D24" s="4" t="inlineStr">
+        <is>
+          <t>Listo (20/10)</t>
+        </is>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1975,8 +1997,10 @@
       <c r="C25" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="D25" s="4" t="s">
-        <v>57</v>
+      <c r="D25" s="4" t="inlineStr">
+        <is>
+          <t>Listo: probado en AWS (falta conectarlo al dashboard)</t>
+        </is>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
docs(nota-2): Product Owner (Abraham) y Scrum Master (Bárbara)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015SVKuYduNdeGeu8Q4SMcKp
</commit_message>
<xml_diff>
--- a/docs/nota-2/Induplac_Roles_Equipo.xlsx
+++ b/docs/nota-2/Induplac_Roles_Equipo.xlsx
@@ -1601,7 +1601,11 @@
       <c r="A13" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="7"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Abraham Castro</t>
+        </is>
+      </c>
       <c r="C13" s="4" t="s">
         <v>36</v>
       </c>
@@ -1610,7 +1614,11 @@
       <c r="A14" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="7"/>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Bárbara Saavedra</t>
+        </is>
+      </c>
       <c r="C14" s="4" t="s">
         <v>38</v>
       </c>

</xml_diff>

<commit_message>
docs(nota-2): fortalezas del equipo (falta la de Lisandra)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015SVKuYduNdeGeu8Q4SMcKp
</commit_message>
<xml_diff>
--- a/docs/nota-2/Induplac_Roles_Equipo.xlsx
+++ b/docs/nota-2/Induplac_Roles_Equipo.xlsx
@@ -1504,7 +1504,11 @@
       <c r="E5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="5"/>
+      <c r="F5" s="5" t="inlineStr">
+        <is>
+          <t>Redes e integración de sistemas: diseña la arquitectura completa (red, broker, Edge y nube) y coordina el repositorio y el trabajo del equipo.</t>
+        </is>
+      </c>
     </row>
     <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
@@ -1522,7 +1526,11 @@
       <c r="E6" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F6" s="5"/>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Electrónica y prototipado IoT: arma el circuito y el firmware del ESP32 (sensores, MQTT con TLS, buffer offline) y resuelve problemas de hardware simulado.</t>
+        </is>
+      </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
@@ -1540,7 +1548,11 @@
       <c r="E7" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="F7" s="5"/>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Pendiente (se define con ella el 21/10).</t>
+        </is>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
@@ -1558,7 +1570,11 @@
       <c r="E8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="F8" s="5"/>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Cloud y seguridad en AWS: configura y administra los servicios (Lambda, RDS, Cognito con MFA, security groups) cuidando el costo y el acceso mínimo.</t>
+        </is>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
@@ -1576,7 +1592,11 @@
       <c r="E9" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="5"/>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Planificación y documentación: organiza el proyecto con RACI, Carta Gantt, Scrum y PMI, y traduce lo técnico a documentos claros.</t>
+        </is>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="6" t="s">

</xml_diff>

<commit_message>
docs(nota-2): Gantt, RACI, tareas, Cloud, Scrum y conclusiones al día con lo construido el 20/10
Propuesta de Bárbara Saavedra. Lo de Lisandra queda pendiente.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EkThzZPLs5mDobXRqBqjok
</commit_message>
<xml_diff>
--- a/docs/nota-2/Induplac_Roles_Equipo.xlsx
+++ b/docs/nota-2/Induplac_Roles_Equipo.xlsx
@@ -22,35 +22,13 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="F5" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Ejemplo de formato: 'Organización y documentación técnica'. Cada integrante escribe la suya.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="249">
   <si>
     <t xml:space="preserve">Induplac IoT — Cargos del equipo (Nota 2, punto 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Autora: Bárbara Saavedra · actualizado 19/10/2026 · Las celdas amarillas las completa cada integrante.</t>
+    <t xml:space="preserve">Autora: Bárbara Saavedra · actualizado 21/10/2026 · Las celdas amarillas las completa cada integrante.</t>
   </si>
   <si>
     <t xml:space="preserve">Integrante</t>
@@ -86,6 +64,9 @@
     <t xml:space="preserve">Todos (transversal)</t>
   </si>
   <si>
+    <t xml:space="preserve">Redes e integración de sistemas: diseña la arquitectura completa (red, broker, Edge y nube) y coordina el repositorio y el trabajo del equipo.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sebastián Fuentes</t>
   </si>
   <si>
@@ -101,6 +82,9 @@
     <t xml:space="preserve">Sprint 2 y 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Electrónica y prototipado IoT: arma el circuito y el firmware del ESP32 (sensores, MQTT con TLS, buffer offline) y resuelve problemas de hardware simulado.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lisandra González</t>
   </si>
   <si>
@@ -116,6 +100,9 @@
     <t xml:space="preserve">Sprint 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Pendiente (se define con ella).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Felipe Murúa</t>
   </si>
   <si>
@@ -128,6 +115,9 @@
     <t xml:space="preserve">backend/, infrastructure/</t>
   </si>
   <si>
+    <t xml:space="preserve">Cloud y seguridad en AWS: configura y administra los servicios (Lambda, RDS, Cognito con MFA, security groups) cuidando el costo y el acceso mínimo.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bárbara Saavedra</t>
   </si>
   <si>
@@ -143,6 +133,9 @@
     <t xml:space="preserve">Sprint 3 e implementación</t>
   </si>
   <si>
+    <t xml:space="preserve">Planificación y documentación: organiza el proyecto con RACI, Carta Gantt, Scrum y PMI, y traduce lo técnico a documentos claros.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Roles Scrum (MVP)</t>
   </si>
   <si>
@@ -209,24 +202,45 @@
     <t xml:space="preserve">Dashboard React con datos simulados y conexión a la API</t>
   </si>
   <si>
+    <t xml:space="preserve">Listo (PR #18)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Edge Gateway en Python: SQLite, intervalos de 15 min, alertas y sincronización</t>
   </si>
   <si>
     <t xml:space="preserve">Backend AWS y base RDS junto a Felipe</t>
   </si>
   <si>
+    <t xml:space="preserve">Listo (PR #16)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login del dashboard con Cognito y MFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En curso (PR #20, falta probar con Felipe)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pipeline DevOps: GitHub Actions (CI en cada PR y despliegue a AWS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listo (PR #21)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Casos de prueba y ensayo de la demo</t>
   </si>
   <si>
+    <t xml:space="preserve">Sebastián</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sketch ESP32 en Wokwi: Local 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sketch ESP32 en Wokwi: Local 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Sebastián</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sketch ESP32 en Wokwi (Local 1 y Local 2)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sensores simulados: CT (kW), caudalímetro (agua) y UV</t>
   </si>
   <si>
@@ -275,13 +289,19 @@
     <t xml:space="preserve">Dashboard publicado en S3</t>
   </si>
   <si>
-    <t xml:space="preserve">RDS PostgreSQL: permisos, umbrales y catálogo (se enciende para la demo)</t>
+    <t xml:space="preserve">RDS PostgreSQL: permisos, umbrales y catálogo + Lambda induplac-config</t>
   </si>
   <si>
     <t xml:space="preserve">Re-deploy de la Lambda con alertas del Edge</t>
   </si>
   <si>
-    <t xml:space="preserve">Cognito con MFA</t>
+    <t xml:space="preserve">Listo (20/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cognito con MFA (user pool, clave temporal y MFA TOTP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listo: probado en AWS</t>
   </si>
   <si>
     <t xml:space="preserve">IAM, TLS, clave de ingesta y cumplimiento Ley 19.628</t>
@@ -321,6 +341,12 @@
   </si>
   <si>
     <t xml:space="preserve">Listo (PR #14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actualización de la Nota 2 con lo construido el 20/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listo (PR #25)</t>
   </si>
   <si>
     <t xml:space="preserve">Capacitación de usuarios del dashboard</t>
@@ -394,7 +420,7 @@
     <t xml:space="preserve">R</t>
   </si>
   <si>
-    <t xml:space="preserve">Backend AWS: API Gateway, Lambda, DynamoDB, RDS PostgreSQL, S3 y reglas de alerta</t>
+    <t xml:space="preserve">Backend AWS: API Gateway, Lambdas (ingesta e induplac-config), DynamoDB, RDS PostgreSQL, S3 y reglas de alerta</t>
   </si>
   <si>
     <t xml:space="preserve">Dashboard React (vistas por sede, alertas, histórico, panel de demo)</t>
@@ -412,7 +438,7 @@
     <t xml:space="preserve">A</t>
   </si>
   <si>
-    <t xml:space="preserve">Documentación, Pull Requests, demo y presentación final</t>
+    <t xml:space="preserve">Documentación, Pull Requests, pipeline DevOps (GitHub Actions), demo y presentación final</t>
   </si>
   <si>
     <t xml:space="preserve">Actividades como R (incluye A/R)</t>
@@ -430,7 +456,7 @@
     <t xml:space="preserve">Inicio del proyecto (lunes semana 1):</t>
   </si>
   <si>
-    <t xml:space="preserve">Cambia esta fecha o las de Inicio/Duración (azul) y todo se recalcula. ■ = semana de trabajo · ◆ = hito</t>
+    <t xml:space="preserve">Cambia esta fecha o las de Inicio/Duración (azul) y todo se recalcula. ■ = semana de trabajo · ◆ = hito · actualizado 21/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -535,7 +561,7 @@
     <t xml:space="preserve">2.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Dashboard React con datos simulados</t>
+    <t xml:space="preserve">Dashboard React (datos simulados y API de AWS)</t>
   </si>
   <si>
     <t xml:space="preserve">2.4</t>
@@ -544,6 +570,9 @@
     <t xml:space="preserve">Backend AWS: API Gateway, Lambda, DynamoDB y S3</t>
   </si>
   <si>
+    <t xml:space="preserve">Felipe y Abraham</t>
+  </si>
+  <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
@@ -553,7 +582,7 @@
     <t xml:space="preserve">3.1</t>
   </si>
   <si>
-    <t xml:space="preserve">ESP32 en Wokwi publicando por MQTT</t>
+    <t xml:space="preserve">ESP32 en Wokwi publicando por MQTT (Local 1 listo; Local 2 pendiente)</t>
   </si>
   <si>
     <t xml:space="preserve">3.2</t>
@@ -571,6 +600,9 @@
     <t xml:space="preserve">3.4</t>
   </si>
   <si>
+    <t xml:space="preserve">Cognito con MFA (probado en AWS; login del dashboard en PR #20)</t>
+  </si>
+  <si>
     <t xml:space="preserve">2.4, 3.3</t>
   </si>
   <si>
@@ -586,6 +618,12 @@
     <t xml:space="preserve">3.1, 3.2, 3.3</t>
   </si>
   <si>
+    <t xml:space="preserve">3.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3, 3.2</t>
+  </si>
+  <si>
     <t xml:space="preserve">4</t>
   </si>
   <si>
@@ -601,6 +639,9 @@
     <t xml:space="preserve">Inicio: validar alcance y criterios de éxito con Induplac</t>
   </si>
   <si>
+    <t xml:space="preserve">Planificado</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.2</t>
   </si>
   <si>
@@ -688,37 +729,52 @@
     <t xml:space="preserve">Hito</t>
   </si>
   <si>
+    <t xml:space="preserve">Cumplido</t>
+  </si>
+  <si>
     <t xml:space="preserve">5.2</t>
   </si>
   <si>
+    <t xml:space="preserve">◆ MVP funcionando de punta a punta (Wokwi → EMQX → Edge → AWS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.3</t>
+  </si>
+  <si>
     <t xml:space="preserve">◆ Demostración del prototipo (miércoles 21/10)</t>
   </si>
   <si>
-    <t xml:space="preserve">5.3</t>
+    <t xml:space="preserve">Hoy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.4</t>
   </si>
   <si>
     <t xml:space="preserve">◆ Acta de inicio con Induplac</t>
   </si>
   <si>
-    <t xml:space="preserve">5.4</t>
+    <t xml:space="preserve">5.5</t>
   </si>
   <si>
     <t xml:space="preserve">◆ Pruebas aprobadas</t>
   </si>
   <si>
-    <t xml:space="preserve">5.5</t>
+    <t xml:space="preserve">5.6</t>
   </si>
   <si>
     <t xml:space="preserve">◆ Puesta en marcha</t>
   </si>
   <si>
-    <t xml:space="preserve">Colores por responsable:</t>
+    <t xml:space="preserve">Colores por responsable (si hay dos, manda el primero):</t>
   </si>
   <si>
     <t xml:space="preserve">Lógica PMI: S1–S3 es el desarrollo del MVP con Scrum (ya en ejecución). S4–S12 es la implementación en Induplac con las 5 fases PMI: inicio (S4), planificación (S5), ejecución (S6–S10), monitoreo y control (transversal) y cierre (S12).</t>
   </si>
   <si>
-    <t xml:space="preserve">Cambio 19/10/2026: RDS PostgreSQL vuelve al MVP (tarea 3.3); se mantiene apagado y se enciende para la demo del miércoles y para configuraciones.</t>
+    <t xml:space="preserve">Estado: Listo / Cumplido = terminado · En curso / Hoy = en desarrollo · Pendiente = atrasado o sin empezar · Planificado = implementación futura.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambios 19/10: RDS PostgreSQL vuelve al MVP (3.3). Cambios 21/10: columna Estado, tarea 3.7 Pipeline DevOps, hito 5.2 MVP de punta a punta (20/10) y responsables compartidos Felipe y Abraham en 2.4, 3.3 y 3.4.</t>
   </si>
 </sst>
 </file>
@@ -730,7 +786,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -794,11 +850,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -976,39 +1027,39 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1016,11 +1067,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1028,19 +1079,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1056,31 +1107,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1488,7 +1539,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1504,114 +1555,104 @@
       <c r="E5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Redes e integración de sistemas: diseña la arquitectura completa (red, broker, Edge y nube) y coordina el repositorio y el trabajo del equipo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F5" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Electrónica y prototipado IoT: arma el circuito y el firmware del ESP32 (sensores, MQTT con TLS, buffer offline) y resuelve problemas de hardware simulado.</t>
-        </is>
+        <v>18</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente (se define con ella el 21/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Cloud y seguridad en AWS: configura y administra los servicios (Lambda, RDS, Cognito con MFA, security groups) cuidando el costo y el acceso mínimo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F8" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Planificación y documentación: organiza el proyecto con RACI, Carta Gantt, Scrum y PMI, y traduce lo técnico a documentos claros.</t>
-        </is>
+        <v>35</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>32</v>
+      <c r="A11" s="7" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
@@ -1619,39 +1660,35 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Abraham Castro</t>
-        </is>
+        <v>40</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>8</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Bárbara Saavedra</t>
-        </is>
+        <v>42</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1662,7 +1699,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1671,7 +1707,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -1682,7 +1718,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1690,570 +1726,602 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #18)</t>
-        </is>
+        <v>18</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #18)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>18</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>58</v>
+      <c r="A10" s="8" t="s">
+        <v>51</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Listo Local 1 (PR #16)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>58</v>
+      <c r="A11" s="8" t="s">
+        <v>51</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
+        <v>18</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
-        <v>64</v>
+      <c r="A15" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>64</v>
+      <c r="A16" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
-        <v>64</v>
+      <c r="A17" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>70</v>
+      <c r="A19" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
-        <v>70</v>
+      <c r="A20" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>70</v>
+      <c r="A21" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
+        <v>56</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Listo (20/10)</t>
-        </is>
+        <v>56</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Listo: probado en AWS (falta conectarlo al dashboard)</t>
-        </is>
+        <v>56</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
-        <v>80</v>
+      <c r="A27" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D27" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
-        <v>80</v>
-      </c>
       <c r="B28" s="4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D28" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
-        <v>80</v>
-      </c>
       <c r="B29" s="4" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>85</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>57</v>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
-        <v>93</v>
+      <c r="A35" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B37" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A37)</f>
-        <v>6</v>
-      </c>
-      <c r="C37" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A37,$D$4:$D$33,"Listo*")</f>
-        <v>1</v>
-      </c>
-      <c r="D37" s="14" t="n">
-        <f aca="false">B37-C37</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B38" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A38)</f>
-        <v>5</v>
-      </c>
-      <c r="C38" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A38,$D$4:$D$33,"Listo*")</f>
-        <v>0</v>
-      </c>
-      <c r="D38" s="14" t="n">
-        <f aca="false">B38-C38</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B39" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A39)</f>
-        <v>4</v>
-      </c>
-      <c r="C39" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A39,$D$4:$D$33,"Listo*")</f>
-        <v>0</v>
-      </c>
-      <c r="D39" s="14" t="n">
-        <f aca="false">B39-C39</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B40" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A40)</f>
-        <v>8</v>
-      </c>
-      <c r="C40" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A40,$D$4:$D$33,"Listo*")</f>
-        <v>4</v>
-      </c>
-      <c r="D40" s="14" t="n">
-        <f aca="false">B40-C40</f>
-        <v>4</v>
+      <c r="B40" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="B41" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A41)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF($A$4:$A$37,A41)</f>
+        <v>8</v>
       </c>
       <c r="C41" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A41,$D$4:$D$33,"Listo*")</f>
-        <v>6</v>
+        <f aca="false">COUNTIFS($A$4:$A$37,A41,$D$4:$D$37,"Listo*")</f>
+        <v>5</v>
       </c>
       <c r="D41" s="14" t="n">
         <f aca="false">B41-C41</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B42" s="14" t="n">
+        <f aca="false">COUNTIF($A$4:$A$37,A42)</f>
+        <v>6</v>
+      </c>
+      <c r="C42" s="14" t="n">
+        <f aca="false">COUNTIFS($A$4:$A$37,A42,$D$4:$D$37,"Listo*")</f>
+        <v>4</v>
+      </c>
+      <c r="D42" s="14" t="n">
+        <f aca="false">B42-C42</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B43" s="14" t="n">
+        <f aca="false">COUNTIF($A$4:$A$37,A43)</f>
+        <v>4</v>
+      </c>
+      <c r="C43" s="14" t="n">
+        <f aca="false">COUNTIFS($A$4:$A$37,A43,$D$4:$D$37,"Listo*")</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="14" t="n">
+        <f aca="false">B43-C43</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B44" s="14" t="n">
+        <f aca="false">COUNTIF($A$4:$A$37,A44)</f>
+        <v>8</v>
+      </c>
+      <c r="C44" s="14" t="n">
+        <f aca="false">COUNTIFS($A$4:$A$37,A44,$D$4:$D$37,"Listo*")</f>
+        <v>7</v>
+      </c>
+      <c r="D44" s="14" t="n">
+        <f aca="false">B44-C44</f>
         <v>1</v>
       </c>
     </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B45" s="14" t="n">
+        <f aca="false">COUNTIF($A$4:$A$37,A45)</f>
+        <v>8</v>
+      </c>
+      <c r="C45" s="14" t="n">
+        <f aca="false">COUNTIFS($A$4:$A$37,A45,$D$4:$D$37,"Listo*")</f>
+        <v>7</v>
+      </c>
+      <c r="D45" s="14" t="n">
+        <f aca="false">B45-C45</f>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D4:D33">
+  <conditionalFormatting sqref="D4:D37">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>LEFT(D4,5)="Listo"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>D4="En curso"</formula>
+      <formula>LEFT(D4,8)="En curso"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2282,38 +2350,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2321,22 +2389,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H5" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C5:G5,"*R*")&gt;=1,COUNTIF(C5:G5,"A*")=1),"OK","Revisar")</f>
@@ -2348,22 +2416,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H6" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C6:G6,"*R*")&gt;=1,COUNTIF(C6:G6,"A*")=1),"OK","Revisar")</f>
@@ -2375,22 +2443,22 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H7" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C7:G7,"*R*")&gt;=1,COUNTIF(C7:G7,"A*")=1),"OK","Revisar")</f>
@@ -2402,22 +2470,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H8" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C8:G8,"*R*")&gt;=1,COUNTIF(C8:G8,"A*")=1),"OK","Revisar")</f>
@@ -2429,22 +2497,22 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H9" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C9:G9,"*R*")&gt;=1,COUNTIF(C9:G9,"A*")=1),"OK","Revisar")</f>
@@ -2456,22 +2524,22 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="H10" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C10:G10,"*R*")&gt;=1,COUNTIF(C10:G10,"A*")=1),"OK","Revisar")</f>
@@ -2483,22 +2551,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H11" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C11:G11,"*R*")&gt;=1,COUNTIF(C11:G11,"A*")=1),"OK","Revisar")</f>
@@ -2510,22 +2578,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="H12" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C12:G12,"*R*")&gt;=1,COUNTIF(C12:G12,"A*")=1),"OK","Revisar")</f>
@@ -2537,49 +2605,49 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="H13" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C13:G13,"*R*")&gt;=1,COUNTIF(C13:G13,"A*")=1),"OK","Revisar")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="H14" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C14:G14,"*R*")&gt;=1,COUNTIF(C14:G14,"A*")=1),"OK","Revisar")</f>
@@ -2588,7 +2656,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="16" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="C16" s="14" t="n">
         <f aca="false">COUNTIF(C5:C14,"*R*")</f>
@@ -2613,7 +2681,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="16" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="C17" s="14" t="n">
         <f aca="false">COUNTIF(C5:C14,"A*")</f>
@@ -2638,7 +2706,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2665,161 +2733,164 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:U51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="9" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="10" style="0" width="6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="E2" s="18" t="n">
         <v>46300</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>126</v>
+      <c r="G2" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>134</v>
+        <v>50</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>145</v>
+        <v>160</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="I5" s="20" t="n">
+        <v>162</v>
+      </c>
+      <c r="J5" s="20" t="n">
         <f aca="false">$E$2+0</f>
         <v>46300</v>
       </c>
-      <c r="J5" s="20" t="n">
+      <c r="K5" s="20" t="n">
         <f aca="false">$E$2+7</f>
         <v>46307</v>
       </c>
-      <c r="K5" s="20" t="n">
+      <c r="L5" s="20" t="n">
         <f aca="false">$E$2+14</f>
         <v>46314</v>
       </c>
-      <c r="L5" s="20" t="n">
+      <c r="M5" s="20" t="n">
         <f aca="false">$E$2+21</f>
         <v>46321</v>
       </c>
-      <c r="M5" s="20" t="n">
+      <c r="N5" s="20" t="n">
         <f aca="false">$E$2+28</f>
         <v>46328</v>
       </c>
-      <c r="N5" s="20" t="n">
+      <c r="O5" s="20" t="n">
         <f aca="false">$E$2+35</f>
         <v>46335</v>
       </c>
-      <c r="O5" s="20" t="n">
+      <c r="P5" s="20" t="n">
         <f aca="false">$E$2+42</f>
         <v>46342</v>
       </c>
-      <c r="P5" s="20" t="n">
+      <c r="Q5" s="20" t="n">
         <f aca="false">$E$2+49</f>
         <v>46349</v>
       </c>
-      <c r="Q5" s="20" t="n">
+      <c r="R5" s="20" t="n">
         <f aca="false">$E$2+56</f>
         <v>46356</v>
       </c>
-      <c r="R5" s="20" t="n">
+      <c r="S5" s="20" t="n">
         <f aca="false">$E$2+63</f>
         <v>46363</v>
       </c>
-      <c r="S5" s="20" t="n">
+      <c r="T5" s="20" t="n">
         <f aca="false">$E$2+70</f>
         <v>46370</v>
       </c>
-      <c r="T5" s="20" t="n">
+      <c r="U5" s="20" t="n">
         <f aca="false">$E$2+77</f>
         <v>46377</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="C6" s="21"/>
       <c r="D6" s="21" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="E6" s="21"/>
       <c r="F6" s="21"/>
@@ -2837,19 +2908,20 @@
       <c r="R6" s="21"/>
       <c r="S6" s="21"/>
       <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="E7" s="22" t="n">
         <v>46300</v>
@@ -2862,15 +2934,14 @@
         <v>46304</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="I7" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E7-6,I$5&lt;=$G7),"■","")</f>
-        <v>■</v>
+        <v>168</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J7" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E7-6,J$5&lt;=$G7),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="K7" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E7-6,K$5&lt;=$G7),"■","")</f>
@@ -2912,19 +2983,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E7-6,T$5&lt;=$G7),"■","")</f>
         <v/>
       </c>
+      <c r="U7" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E7-6,U$5&lt;=$G7),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" s="22" t="n">
         <v>46307</v>
@@ -2937,15 +3012,14 @@
         <v>46318</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="I8" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E8-6,I$5&lt;=$G8),"■","")</f>
-        <v/>
+        <v>166</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J8" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E8-6,J$5&lt;=$G8),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K8" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E8-6,K$5&lt;=$G8),"■","")</f>
@@ -2953,7 +3027,7 @@
       </c>
       <c r="L8" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E8-6,L$5&lt;=$G8),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M8" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E8-6,M$5&lt;=$G8),"■","")</f>
@@ -2987,17 +3061,21 @@
         <f aca="false">IF(AND(T$5&gt;=$E8-6,T$5&lt;=$G8),"■","")</f>
         <v/>
       </c>
+      <c r="U8" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E8-6,U$5&lt;=$G8),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="C9" s="21"/>
       <c r="D9" s="21" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E9" s="21"/>
       <c r="F9" s="21"/>
@@ -3015,19 +3093,20 @@
       <c r="R9" s="21"/>
       <c r="S9" s="21"/>
       <c r="T9" s="21"/>
+      <c r="U9" s="21"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E10" s="22" t="n">
         <v>46307</v>
@@ -3040,19 +3119,18 @@
         <v>46311</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="I10" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E10-6,I$5&lt;=$G10),"■","")</f>
-        <v/>
+        <v>166</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J10" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E10-6,J$5&lt;=$G10),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K10" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E10-6,K$5&lt;=$G10),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L10" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E10-6,L$5&lt;=$G10),"■","")</f>
@@ -3090,19 +3168,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E10-6,T$5&lt;=$G10),"■","")</f>
         <v/>
       </c>
+      <c r="U10" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E10-6,U$5&lt;=$G10),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E11" s="22" t="n">
         <v>46307</v>
@@ -3115,19 +3197,18 @@
         <v>46311</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="I11" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E11-6,I$5&lt;=$G11),"■","")</f>
-        <v/>
+        <v>173</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J11" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E11-6,J$5&lt;=$G11),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K11" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E11-6,K$5&lt;=$G11),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L11" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E11-6,L$5&lt;=$G11),"■","")</f>
@@ -3165,19 +3246,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E11-6,T$5&lt;=$G11),"■","")</f>
         <v/>
       </c>
+      <c r="U11" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E11-6,U$5&lt;=$G11),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" s="22" t="n">
         <v>46307</v>
@@ -3190,15 +3275,14 @@
         <v>46318</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="I12" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E12-6,I$5&lt;=$G12),"■","")</f>
-        <v/>
+        <v>173</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J12" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E12-6,J$5&lt;=$G12),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K12" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E12-6,K$5&lt;=$G12),"■","")</f>
@@ -3206,7 +3290,7 @@
       </c>
       <c r="L12" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E12-6,L$5&lt;=$G12),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M12" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E12-6,M$5&lt;=$G12),"■","")</f>
@@ -3240,19 +3324,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E12-6,T$5&lt;=$G12),"■","")</f>
         <v/>
       </c>
+      <c r="U12" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E12-6,U$5&lt;=$G12),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E13" s="22" t="n">
         <v>46307</v>
@@ -3265,15 +3353,14 @@
         <v>46318</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="I13" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E13-6,I$5&lt;=$G13),"■","")</f>
-        <v/>
+        <v>173</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J13" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E13-6,J$5&lt;=$G13),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K13" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E13-6,K$5&lt;=$G13),"■","")</f>
@@ -3281,7 +3368,7 @@
       </c>
       <c r="L13" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E13-6,L$5&lt;=$G13),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M13" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E13-6,M$5&lt;=$G13),"■","")</f>
@@ -3315,17 +3402,21 @@
         <f aca="false">IF(AND(T$5&gt;=$E13-6,T$5&lt;=$G13),"■","")</f>
         <v/>
       </c>
+      <c r="U13" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E13-6,U$5&lt;=$G13),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="C14" s="21"/>
       <c r="D14" s="21" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E14" s="21"/>
       <c r="F14" s="21"/>
@@ -3343,19 +3434,20 @@
       <c r="R14" s="21"/>
       <c r="S14" s="21"/>
       <c r="T14" s="21"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U14" s="21"/>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E15" s="22" t="n">
         <v>46307</v>
@@ -3368,15 +3460,14 @@
         <v>46318</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="I15" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E15-6,I$5&lt;=$G15),"■","")</f>
-        <v/>
+        <v>175</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="J15" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E15-6,J$5&lt;=$G15),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K15" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E15-6,K$5&lt;=$G15),"■","")</f>
@@ -3384,7 +3475,7 @@
       </c>
       <c r="L15" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E15-6,L$5&lt;=$G15),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M15" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E15-6,M$5&lt;=$G15),"■","")</f>
@@ -3418,19 +3509,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E15-6,T$5&lt;=$G15),"■","")</f>
         <v/>
       </c>
+      <c r="U15" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E15-6,U$5&lt;=$G15),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E16" s="22" t="n">
         <v>46307</v>
@@ -3443,15 +3538,14 @@
         <v>46318</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="I16" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E16-6,I$5&lt;=$G16),"■","")</f>
-        <v/>
+        <v>187</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J16" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E16-6,J$5&lt;=$G16),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K16" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E16-6,K$5&lt;=$G16),"■","")</f>
@@ -3459,7 +3553,7 @@
       </c>
       <c r="L16" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E16-6,L$5&lt;=$G16),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M16" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E16-6,M$5&lt;=$G16),"■","")</f>
@@ -3493,19 +3587,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E16-6,T$5&lt;=$G16),"■","")</f>
         <v/>
       </c>
+      <c r="U16" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E16-6,U$5&lt;=$G16),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E17" s="22" t="n">
         <v>46314</v>
@@ -3518,11 +3616,10 @@
         <v>46318</v>
       </c>
       <c r="H17" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="I17" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E17-6,I$5&lt;=$G17),"■","")</f>
-        <v/>
+        <v>178</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J17" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E17-6,J$5&lt;=$G17),"■","")</f>
@@ -3530,11 +3627,11 @@
       </c>
       <c r="K17" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E17-6,K$5&lt;=$G17),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="L17" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E17-6,L$5&lt;=$G17),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M17" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E17-6,M$5&lt;=$G17),"■","")</f>
@@ -3568,19 +3665,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E17-6,T$5&lt;=$G17),"■","")</f>
         <v/>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U17" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E17-6,U$5&lt;=$G17),"■","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>172</v>
+        <v>189</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>78</v>
+        <v>190</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E18" s="22" t="n">
         <v>46314</v>
@@ -3593,11 +3694,10 @@
         <v>46318</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="I18" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E18-6,I$5&lt;=$G18),"■","")</f>
-        <v/>
+        <v>191</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="J18" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E18-6,J$5&lt;=$G18),"■","")</f>
@@ -3605,11 +3705,11 @@
       </c>
       <c r="K18" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E18-6,K$5&lt;=$G18),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="L18" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E18-6,L$5&lt;=$G18),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M18" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E18-6,M$5&lt;=$G18),"■","")</f>
@@ -3643,19 +3743,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E18-6,T$5&lt;=$G18),"■","")</f>
         <v/>
       </c>
+      <c r="U18" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E18-6,U$5&lt;=$G18),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E19" s="22" t="n">
         <v>46314</v>
@@ -3668,11 +3772,10 @@
         <v>46318</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="I19" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E19-6,I$5&lt;=$G19),"■","")</f>
-        <v/>
+        <v>185</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>71</v>
       </c>
       <c r="J19" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E19-6,J$5&lt;=$G19),"■","")</f>
@@ -3680,11 +3783,11 @@
       </c>
       <c r="K19" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E19-6,K$5&lt;=$G19),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="L19" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E19-6,L$5&lt;=$G19),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M19" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E19-6,M$5&lt;=$G19),"■","")</f>
@@ -3718,19 +3821,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E19-6,T$5&lt;=$G19),"■","")</f>
         <v/>
       </c>
+      <c r="U19" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E19-6,U$5&lt;=$G19),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E20" s="22" t="n">
         <v>46314</v>
@@ -3743,11 +3850,10 @@
         <v>46318</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="I20" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E20-6,I$5&lt;=$G20),"■","")</f>
-        <v/>
+        <v>195</v>
+      </c>
+      <c r="I20" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="J20" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E20-6,J$5&lt;=$G20),"■","")</f>
@@ -3755,11 +3861,11 @@
       </c>
       <c r="K20" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E20-6,K$5&lt;=$G20),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="L20" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E20-6,L$5&lt;=$G20),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M20" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E20-6,M$5&lt;=$G20),"■","")</f>
@@ -3793,139 +3899,146 @@
         <f aca="false">IF(AND(T$5&gt;=$E20-6,T$5&lt;=$G20),"■","")</f>
         <v/>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>179</v>
-      </c>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21" t="s">
-        <v>180</v>
-      </c>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-      <c r="N21" s="21"/>
-      <c r="O21" s="21"/>
-      <c r="P21" s="21"/>
-      <c r="Q21" s="21"/>
-      <c r="R21" s="21"/>
-      <c r="S21" s="21"/>
-      <c r="T21" s="21"/>
+      <c r="U20" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E20-6,U$5&lt;=$G20),"■","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="22" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F21" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <f aca="false">E21+F21*7-3</f>
+        <v>46318</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="J21" s="25" t="str">
+        <f aca="false">IF(AND(J$5&gt;=$E21-6,J$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="K21" s="25" t="str">
+        <f aca="false">IF(AND(K$5&gt;=$E21-6,K$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="L21" s="25" t="str">
+        <f aca="false">IF(AND(L$5&gt;=$E21-6,L$5&lt;=$G21),"■","")</f>
+        <v>■</v>
+      </c>
+      <c r="M21" s="25" t="str">
+        <f aca="false">IF(AND(M$5&gt;=$E21-6,M$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="N21" s="25" t="str">
+        <f aca="false">IF(AND(N$5&gt;=$E21-6,N$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="O21" s="25" t="str">
+        <f aca="false">IF(AND(O$5&gt;=$E21-6,O$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="P21" s="25" t="str">
+        <f aca="false">IF(AND(P$5&gt;=$E21-6,P$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="Q21" s="25" t="str">
+        <f aca="false">IF(AND(Q$5&gt;=$E21-6,Q$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="R21" s="25" t="str">
+        <f aca="false">IF(AND(R$5&gt;=$E21-6,R$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="S21" s="25" t="str">
+        <f aca="false">IF(AND(S$5&gt;=$E21-6,S$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="T21" s="25" t="str">
+        <f aca="false">IF(AND(T$5&gt;=$E21-6,T$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="U21" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E21-6,U$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="E22" s="22" t="n">
+      <c r="A22" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>199</v>
+      </c>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="21"/>
+      <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="21"/>
+      <c r="P22" s="21"/>
+      <c r="Q22" s="21"/>
+      <c r="R22" s="21"/>
+      <c r="S22" s="21"/>
+      <c r="T22" s="21"/>
+      <c r="U22" s="21"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E23" s="22" t="n">
         <v>46321</v>
-      </c>
-      <c r="F22" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="24" t="n">
-        <f aca="false">E22+F22*7-3</f>
-        <v>46325</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="I22" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E22-6,I$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="J22" s="25" t="str">
-        <f aca="false">IF(AND(J$5&gt;=$E22-6,J$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="K22" s="25" t="str">
-        <f aca="false">IF(AND(K$5&gt;=$E22-6,K$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="L22" s="25" t="str">
-        <f aca="false">IF(AND(L$5&gt;=$E22-6,L$5&lt;=$G22),"■","")</f>
-        <v>■</v>
-      </c>
-      <c r="M22" s="25" t="str">
-        <f aca="false">IF(AND(M$5&gt;=$E22-6,M$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="N22" s="25" t="str">
-        <f aca="false">IF(AND(N$5&gt;=$E22-6,N$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="O22" s="25" t="str">
-        <f aca="false">IF(AND(O$5&gt;=$E22-6,O$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="P22" s="25" t="str">
-        <f aca="false">IF(AND(P$5&gt;=$E22-6,P$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="Q22" s="25" t="str">
-        <f aca="false">IF(AND(Q$5&gt;=$E22-6,Q$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="R22" s="25" t="str">
-        <f aca="false">IF(AND(R$5&gt;=$E22-6,R$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="S22" s="25" t="str">
-        <f aca="false">IF(AND(S$5&gt;=$E22-6,S$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="T22" s="25" t="str">
-        <f aca="false">IF(AND(T$5&gt;=$E22-6,T$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E23" s="22" t="n">
-        <v>46328</v>
       </c>
       <c r="F23" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="24" t="n">
         <f aca="false">E23+F23*7-3</f>
-        <v>46332</v>
+        <v>46325</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="I23" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E23-6,I$5&lt;=$G23),"■","")</f>
-        <v/>
+        <v>194</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J23" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E23-6,J$5&lt;=$G23),"■","")</f>
@@ -3971,36 +4084,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E23-6,T$5&lt;=$G23),"■","")</f>
         <v/>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U23" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E23-6,U$5&lt;=$G23),"■","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>188</v>
+        <v>206</v>
       </c>
       <c r="E24" s="22" t="n">
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" s="24" t="n">
         <f aca="false">E24+F24*7-3</f>
-        <v>46346</v>
+        <v>46332</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="I24" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E24-6,I$5&lt;=$G24),"■","")</f>
-        <v/>
+        <v>201</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J24" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E24-6,J$5&lt;=$G24),"■","")</f>
@@ -4024,7 +4140,7 @@
       </c>
       <c r="O24" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E24-6,O$5&lt;=$G24),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="P24" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E24-6,P$5&lt;=$G24),"■","")</f>
@@ -4046,19 +4162,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E24-6,T$5&lt;=$G24),"■","")</f>
         <v/>
       </c>
+      <c r="U24" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E24-6,U$5&lt;=$G24),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>190</v>
+        <v>208</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="E25" s="22" t="n">
         <v>46335</v>
@@ -4071,11 +4191,10 @@
         <v>46346</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="I25" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E25-6,I$5&lt;=$G25),"■","")</f>
-        <v/>
+        <v>204</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J25" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E25-6,J$5&lt;=$G25),"■","")</f>
@@ -4095,7 +4214,7 @@
       </c>
       <c r="N25" s="25" t="str">
         <f aca="false">IF(AND(N$5&gt;=$E25-6,N$5&lt;=$G25),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="O25" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E25-6,O$5&lt;=$G25),"■","")</f>
@@ -4103,7 +4222,7 @@
       </c>
       <c r="P25" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E25-6,P$5&lt;=$G25),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="Q25" s="25" t="str">
         <f aca="false">IF(AND(Q$5&gt;=$E25-6,Q$5&lt;=$G25),"■","")</f>
@@ -4121,19 +4240,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E25-6,T$5&lt;=$G25),"■","")</f>
         <v/>
       </c>
+      <c r="U25" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E25-6,U$5&lt;=$G25),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="E26" s="22" t="n">
         <v>46335</v>
@@ -4146,11 +4269,10 @@
         <v>46346</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="I26" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E26-6,I$5&lt;=$G26),"■","")</f>
-        <v/>
+        <v>204</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J26" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E26-6,J$5&lt;=$G26),"■","")</f>
@@ -4170,7 +4292,7 @@
       </c>
       <c r="N26" s="25" t="str">
         <f aca="false">IF(AND(N$5&gt;=$E26-6,N$5&lt;=$G26),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="O26" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E26-6,O$5&lt;=$G26),"■","")</f>
@@ -4178,7 +4300,7 @@
       </c>
       <c r="P26" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E26-6,P$5&lt;=$G26),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="Q26" s="25" t="str">
         <f aca="false">IF(AND(Q$5&gt;=$E26-6,Q$5&lt;=$G26),"■","")</f>
@@ -4196,36 +4318,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E26-6,T$5&lt;=$G26),"■","")</f>
         <v/>
       </c>
+      <c r="U26" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E26-6,U$5&lt;=$G26),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="E27" s="22" t="n">
-        <v>46349</v>
+        <v>46335</v>
       </c>
       <c r="F27" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G27" s="24" t="n">
         <f aca="false">E27+F27*7-3</f>
-        <v>46353</v>
+        <v>46346</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>196</v>
-      </c>
-      <c r="I27" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E27-6,I$5&lt;=$G27),"■","")</f>
-        <v/>
+        <v>204</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J27" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E27-6,J$5&lt;=$G27),"■","")</f>
@@ -4249,7 +4374,7 @@
       </c>
       <c r="O27" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E27-6,O$5&lt;=$G27),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="P27" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E27-6,P$5&lt;=$G27),"■","")</f>
@@ -4271,36 +4396,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E27-6,T$5&lt;=$G27),"■","")</f>
         <v/>
       </c>
+      <c r="U27" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E27-6,U$5&lt;=$G27),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>188</v>
+        <v>216</v>
       </c>
       <c r="E28" s="22" t="n">
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="F28" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="24" t="n">
         <f aca="false">E28+F28*7-3</f>
-        <v>46360</v>
+        <v>46353</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="I28" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E28-6,I$5&lt;=$G28),"■","")</f>
-        <v/>
+        <v>217</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J28" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E28-6,J$5&lt;=$G28),"■","")</f>
@@ -4346,36 +4474,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E28-6,T$5&lt;=$G28),"■","")</f>
         <v/>
       </c>
+      <c r="U28" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E28-6,U$5&lt;=$G28),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="E29" s="22" t="n">
-        <v>46363</v>
+        <v>46356</v>
       </c>
       <c r="F29" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G29" s="24" t="n">
         <f aca="false">E29+F29*7-3</f>
-        <v>46367</v>
+        <v>46360</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>197</v>
-      </c>
-      <c r="I29" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E29-6,I$5&lt;=$G29),"■","")</f>
-        <v/>
+        <v>214</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J29" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E29-6,J$5&lt;=$G29),"■","")</f>
@@ -4421,36 +4552,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E29-6,T$5&lt;=$G29),"■","")</f>
         <v/>
       </c>
+      <c r="U29" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E29-6,U$5&lt;=$G29),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="E30" s="22" t="n">
-        <v>46321</v>
+        <v>46363</v>
       </c>
       <c r="F30" s="23" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G30" s="24" t="n">
         <f aca="false">E30+F30*7-3</f>
-        <v>46374</v>
+        <v>46367</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="I30" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E30-6,I$5&lt;=$G30),"■","")</f>
-        <v/>
+        <v>218</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J30" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E30-6,J$5&lt;=$G30),"■","")</f>
@@ -4462,31 +4596,31 @@
       </c>
       <c r="L30" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E30-6,L$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="M30" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E30-6,M$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="N30" s="25" t="str">
         <f aca="false">IF(AND(N$5&gt;=$E30-6,N$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="O30" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E30-6,O$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="P30" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E30-6,P$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="Q30" s="25" t="str">
         <f aca="false">IF(AND(Q$5&gt;=$E30-6,Q$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="R30" s="25" t="str">
         <f aca="false">IF(AND(R$5&gt;=$E30-6,R$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="S30" s="25" t="str">
         <f aca="false">IF(AND(S$5&gt;=$E30-6,S$5&lt;=$G30),"■","")</f>
@@ -4496,36 +4630,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E30-6,T$5&lt;=$G30),"■","")</f>
         <v/>
       </c>
+      <c r="U30" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E30-6,U$5&lt;=$G30),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="E31" s="22" t="n">
-        <v>46377</v>
+        <v>46321</v>
       </c>
       <c r="F31" s="23" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G31" s="24" t="n">
         <f aca="false">E31+F31*7-3</f>
-        <v>46381</v>
+        <v>46374</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="I31" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E31-6,I$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>168</v>
+      </c>
+      <c r="I31" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J31" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E31-6,J$5&lt;=$G31),"■","")</f>
@@ -4541,169 +4678,176 @@
       </c>
       <c r="M31" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E31-6,M$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="N31" s="25" t="str">
         <f aca="false">IF(AND(N$5&gt;=$E31-6,N$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="O31" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E31-6,O$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="P31" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E31-6,P$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="Q31" s="25" t="str">
         <f aca="false">IF(AND(Q$5&gt;=$E31-6,Q$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="R31" s="25" t="str">
         <f aca="false">IF(AND(R$5&gt;=$E31-6,R$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="S31" s="25" t="str">
         <f aca="false">IF(AND(S$5&gt;=$E31-6,S$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="T31" s="25" t="str">
         <f aca="false">IF(AND(T$5&gt;=$E31-6,T$5&lt;=$G31),"■","")</f>
         <v>■</v>
       </c>
+      <c r="U31" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E31-6,U$5&lt;=$G31),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="21"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="21"/>
-      <c r="O32" s="21"/>
-      <c r="P32" s="21"/>
-      <c r="Q32" s="21"/>
-      <c r="R32" s="21"/>
-      <c r="S32" s="21"/>
-      <c r="T32" s="21"/>
+      <c r="A32" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E32" s="22" t="n">
+        <v>46377</v>
+      </c>
+      <c r="F32" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <f aca="false">E32+F32*7-3</f>
+        <v>46381</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="J32" s="25" t="str">
+        <f aca="false">IF(AND(J$5&gt;=$E32-6,J$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="K32" s="25" t="str">
+        <f aca="false">IF(AND(K$5&gt;=$E32-6,K$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="L32" s="25" t="str">
+        <f aca="false">IF(AND(L$5&gt;=$E32-6,L$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="M32" s="25" t="str">
+        <f aca="false">IF(AND(M$5&gt;=$E32-6,M$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="N32" s="25" t="str">
+        <f aca="false">IF(AND(N$5&gt;=$E32-6,N$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="O32" s="25" t="str">
+        <f aca="false">IF(AND(O$5&gt;=$E32-6,O$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="P32" s="25" t="str">
+        <f aca="false">IF(AND(P$5&gt;=$E32-6,P$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="Q32" s="25" t="str">
+        <f aca="false">IF(AND(Q$5&gt;=$E32-6,Q$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="R32" s="25" t="str">
+        <f aca="false">IF(AND(R$5&gt;=$E32-6,R$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="S32" s="25" t="str">
+        <f aca="false">IF(AND(S$5&gt;=$E32-6,S$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="T32" s="25" t="str">
+        <f aca="false">IF(AND(T$5&gt;=$E32-6,T$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="U32" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E32-6,U$5&lt;=$G32),"■","")</f>
+        <v>■</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
-        <v>208</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="E33" s="22" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F33" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="24" t="n">
-        <f aca="false">E33</f>
-        <v>46311</v>
-      </c>
-      <c r="H33" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="I33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=I$5,$E33&lt;I$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="J33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=J$5,$E33&lt;J$5+7),"◆","")</f>
-        <v>◆</v>
-      </c>
-      <c r="K33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=K$5,$E33&lt;K$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="L33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=L$5,$E33&lt;L$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="M33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=M$5,$E33&lt;M$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="N33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=N$5,$E33&lt;N$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="O33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=O$5,$E33&lt;O$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="P33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=P$5,$E33&lt;P$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="Q33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=Q$5,$E33&lt;Q$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="R33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=R$5,$E33&lt;R$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="S33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=S$5,$E33&lt;S$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="T33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=T$5,$E33&lt;T$5+7),"◆","")</f>
-        <v/>
-      </c>
+      <c r="A33" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+      <c r="M33" s="21"/>
+      <c r="N33" s="21"/>
+      <c r="O33" s="21"/>
+      <c r="P33" s="21"/>
+      <c r="Q33" s="21"/>
+      <c r="R33" s="21"/>
+      <c r="S33" s="21"/>
+      <c r="T33" s="21"/>
+      <c r="U33" s="21"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>213</v>
+        <v>230</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="E34" s="22" t="n">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="F34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="24" t="n">
         <f aca="false">E34</f>
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="I34" s="25" t="str">
-        <f aca="false">IF(AND($E34&gt;=I$5,$E34&lt;I$5+7),"◆","")</f>
-        <v/>
+        <v>187</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>233</v>
       </c>
       <c r="J34" s="25" t="str">
         <f aca="false">IF(AND($E34&gt;=J$5,$E34&lt;J$5+7),"◆","")</f>
@@ -4749,36 +4893,39 @@
         <f aca="false">IF(AND($E34&gt;=T$5,$E34&lt;T$5+7),"◆","")</f>
         <v/>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U34" s="25" t="str">
+        <f aca="false">IF(AND($E34&gt;=U$5,$E34&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>215</v>
+        <v>235</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="E35" s="22" t="n">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="F35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="24" t="n">
         <f aca="false">E35</f>
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="I35" s="25" t="str">
-        <f aca="false">IF(AND($E35&gt;=I$5,$E35&lt;I$5+7),"◆","")</f>
-        <v/>
+        <v>195</v>
+      </c>
+      <c r="I35" s="14" t="s">
+        <v>233</v>
       </c>
       <c r="J35" s="25" t="str">
         <f aca="false">IF(AND($E35&gt;=J$5,$E35&lt;J$5+7),"◆","")</f>
@@ -4824,36 +4971,39 @@
         <f aca="false">IF(AND($E35&gt;=T$5,$E35&lt;T$5+7),"◆","")</f>
         <v/>
       </c>
+      <c r="U35" s="25" t="str">
+        <f aca="false">IF(AND($E35&gt;=U$5,$E35&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>216</v>
+        <v>236</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>217</v>
+        <v>237</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="E36" s="22" t="n">
-        <v>46353</v>
+        <v>46316</v>
       </c>
       <c r="F36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="24" t="n">
         <f aca="false">E36</f>
-        <v>46353</v>
+        <v>46316</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="I36" s="25" t="str">
-        <f aca="false">IF(AND($E36&gt;=I$5,$E36&lt;I$5+7),"◆","")</f>
-        <v/>
+        <v>194</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>238</v>
       </c>
       <c r="J36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=J$5,$E36&lt;J$5+7),"◆","")</f>
@@ -4865,7 +5015,7 @@
       </c>
       <c r="L36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=L$5,$E36&lt;L$5+7),"◆","")</f>
-        <v/>
+        <v>◆</v>
       </c>
       <c r="M36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=M$5,$E36&lt;M$5+7),"◆","")</f>
@@ -4881,7 +5031,7 @@
       </c>
       <c r="P36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=P$5,$E36&lt;P$5+7),"◆","")</f>
-        <v>◆</v>
+        <v/>
       </c>
       <c r="Q36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=Q$5,$E36&lt;Q$5+7),"◆","")</f>
@@ -4899,36 +5049,39 @@
         <f aca="false">IF(AND($E36&gt;=T$5,$E36&lt;T$5+7),"◆","")</f>
         <v/>
       </c>
+      <c r="U36" s="25" t="str">
+        <f aca="false">IF(AND($E36&gt;=U$5,$E36&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="E37" s="22" t="n">
-        <v>46370</v>
+        <v>46325</v>
       </c>
       <c r="F37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="24" t="n">
         <f aca="false">E37</f>
-        <v>46370</v>
+        <v>46325</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="I37" s="25" t="str">
-        <f aca="false">IF(AND($E37&gt;=I$5,$E37&lt;I$5+7),"◆","")</f>
-        <v/>
+        <v>201</v>
+      </c>
+      <c r="I37" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=J$5,$E37&lt;J$5+7),"◆","")</f>
@@ -4944,7 +5097,7 @@
       </c>
       <c r="M37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=M$5,$E37&lt;M$5+7),"◆","")</f>
-        <v/>
+        <v>◆</v>
       </c>
       <c r="N37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=N$5,$E37&lt;N$5+7),"◆","")</f>
@@ -4968,117 +5121,321 @@
       </c>
       <c r="S37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=S$5,$E37&lt;S$5+7),"◆","")</f>
-        <v>◆</v>
+        <v/>
       </c>
       <c r="T37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=T$5,$E37&lt;T$5+7),"◆","")</f>
         <v/>
       </c>
+      <c r="U37" s="25" t="str">
+        <f aca="false">IF(AND($E37&gt;=U$5,$E37&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E38" s="22" t="n">
+        <v>46353</v>
+      </c>
+      <c r="F38" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <f aca="false">E38</f>
+        <v>46353</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="J38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=J$5,$E38&lt;J$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="K38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=K$5,$E38&lt;K$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="L38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=L$5,$E38&lt;L$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="M38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=M$5,$E38&lt;M$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="N38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=N$5,$E38&lt;N$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="O38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=O$5,$E38&lt;O$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="P38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=P$5,$E38&lt;P$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="Q38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=Q$5,$E38&lt;Q$5+7),"◆","")</f>
+        <v>◆</v>
+      </c>
+      <c r="R38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=R$5,$E38&lt;R$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="S38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=S$5,$E38&lt;S$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="T38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=T$5,$E38&lt;T$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="U38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=U$5,$E38&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="16" t="s">
+      <c r="A39" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E39" s="22" t="n">
+        <v>46370</v>
+      </c>
+      <c r="F39" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <f aca="false">E39</f>
+        <v>46370</v>
+      </c>
+      <c r="H39" s="14" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="26" t="s">
-        <v>46</v>
+      <c r="I39" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="J39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=J$5,$E39&lt;J$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="K39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=K$5,$E39&lt;K$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="L39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=L$5,$E39&lt;L$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="M39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=M$5,$E39&lt;M$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="N39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=N$5,$E39&lt;N$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="O39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=O$5,$E39&lt;O$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="P39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=P$5,$E39&lt;P$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="Q39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=Q$5,$E39&lt;Q$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="R39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=R$5,$E39&lt;R$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="S39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=S$5,$E39&lt;S$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="T39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=T$5,$E39&lt;T$5+7),"◆","")</f>
+        <v>◆</v>
+      </c>
+      <c r="U39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=U$5,$E39&lt;U$5+7),"◆","")</f>
+        <v/>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="27" t="s">
-        <v>58</v>
+      <c r="B41" s="16" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="28" t="s">
-        <v>64</v>
+      <c r="B42" s="26" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="29" t="s">
-        <v>70</v>
+      <c r="B43" s="27" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="30" t="s">
-        <v>80</v>
+      <c r="B44" s="28" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="31" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="32" t="s">
-        <v>221</v>
-      </c>
-      <c r="C47" s="32"/>
-      <c r="D47" s="32"/>
-      <c r="E47" s="32"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
-      <c r="H47" s="32"/>
-      <c r="I47" s="32"/>
-      <c r="J47" s="32"/>
-      <c r="K47" s="32"/>
-      <c r="L47" s="32"/>
-      <c r="M47" s="32"/>
-      <c r="N47" s="32"/>
-      <c r="O47" s="32"/>
-      <c r="P47" s="32"/>
-      <c r="Q47" s="32"/>
-      <c r="R47" s="32"/>
-      <c r="S47" s="32"/>
-      <c r="T47" s="32"/>
-    </row>
-    <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="32" t="s">
-        <v>222</v>
-      </c>
-      <c r="C48" s="32"/>
-      <c r="D48" s="32"/>
-      <c r="E48" s="32"/>
-      <c r="F48" s="32"/>
-      <c r="G48" s="32"/>
-      <c r="H48" s="32"/>
-      <c r="I48" s="32"/>
-      <c r="J48" s="32"/>
-      <c r="K48" s="32"/>
-      <c r="L48" s="32"/>
-      <c r="M48" s="32"/>
-      <c r="N48" s="32"/>
-      <c r="O48" s="32"/>
-      <c r="P48" s="32"/>
-      <c r="Q48" s="32"/>
-      <c r="R48" s="32"/>
-      <c r="S48" s="32"/>
-      <c r="T48" s="32"/>
+      <c r="B45" s="29" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="30" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="31" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B49" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="C49" s="32"/>
+      <c r="D49" s="32"/>
+      <c r="E49" s="32"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="32"/>
+      <c r="H49" s="32"/>
+      <c r="I49" s="32"/>
+      <c r="J49" s="32"/>
+      <c r="K49" s="32"/>
+      <c r="L49" s="32"/>
+      <c r="M49" s="32"/>
+      <c r="N49" s="32"/>
+      <c r="O49" s="32"/>
+      <c r="P49" s="32"/>
+      <c r="Q49" s="32"/>
+      <c r="R49" s="32"/>
+      <c r="S49" s="32"/>
+      <c r="T49" s="32"/>
+      <c r="U49" s="32"/>
+    </row>
+    <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B50" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="C50" s="32"/>
+      <c r="D50" s="32"/>
+      <c r="E50" s="32"/>
+      <c r="F50" s="32"/>
+      <c r="G50" s="32"/>
+      <c r="H50" s="32"/>
+      <c r="I50" s="32"/>
+      <c r="J50" s="32"/>
+      <c r="K50" s="32"/>
+      <c r="L50" s="32"/>
+      <c r="M50" s="32"/>
+      <c r="N50" s="32"/>
+      <c r="O50" s="32"/>
+      <c r="P50" s="32"/>
+      <c r="Q50" s="32"/>
+      <c r="R50" s="32"/>
+      <c r="S50" s="32"/>
+      <c r="T50" s="32"/>
+      <c r="U50" s="32"/>
+    </row>
+    <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B51" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="C51" s="32"/>
+      <c r="D51" s="32"/>
+      <c r="E51" s="32"/>
+      <c r="F51" s="32"/>
+      <c r="G51" s="32"/>
+      <c r="H51" s="32"/>
+      <c r="I51" s="32"/>
+      <c r="J51" s="32"/>
+      <c r="K51" s="32"/>
+      <c r="L51" s="32"/>
+      <c r="M51" s="32"/>
+      <c r="N51" s="32"/>
+      <c r="O51" s="32"/>
+      <c r="P51" s="32"/>
+      <c r="Q51" s="32"/>
+      <c r="R51" s="32"/>
+      <c r="S51" s="32"/>
+      <c r="T51" s="32"/>
+      <c r="U51" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B47:T47"/>
-    <mergeCell ref="B48:T48"/>
+  <mergeCells count="3">
+    <mergeCell ref="B49:U49"/>
+    <mergeCell ref="B50:U50"/>
+    <mergeCell ref="B51:U51"/>
   </mergeCells>
-  <conditionalFormatting sqref="I6:T37">
+  <conditionalFormatting sqref="J6:U39">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>AND(I6&lt;&gt;"",$C6="Abraham")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,7)="Abraham")</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(I6&lt;&gt;"",$C6="Sebastián")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,9)="Sebastián")</formula>
     </cfRule>
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
-      <formula>AND(I6&lt;&gt;"",$C6="Lisandra")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,8)="Lisandra")</formula>
     </cfRule>
     <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
-      <formula>AND(I6&lt;&gt;"",$C6="Felipe")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,6)="Felipe")</formula>
     </cfRule>
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
-      <formula>AND(I6&lt;&gt;"",$C6="Bárbara")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,7)="Bárbara")</formula>
     </cfRule>
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
-      <formula>AND(I6&lt;&gt;"",$C6="Equipo")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,6)="Equipo")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:I39">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>I6="Listo"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>I6="Cumplido"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>I6="En curso"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>I6="Hoy"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>I6="Pendiente"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
docs(nota-2): Gantt, RACI y documentos de Bárbara al día con lo del 20/10 (#25)
Aceptado a pedido de Bárbara (21/10/2026).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EkThzZPLs5mDobXRqBqjok
</commit_message>
<xml_diff>
--- a/docs/nota-2/Induplac_Roles_Equipo.xlsx
+++ b/docs/nota-2/Induplac_Roles_Equipo.xlsx
@@ -22,35 +22,13 @@
 </workbook>
 </file>
 
-<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <authors>
-    <author>Unknown Author</author>
-  </authors>
-  <commentList>
-    <comment ref="F5" authorId="0">
-      <text>
-        <r>
-          <rPr>
-            <sz val="10"/>
-            <rFont val="Arial"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">Ejemplo de formato: 'Organización y documentación técnica'. Cada integrante escribe la suya.</t>
-        </r>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="435" uniqueCount="223">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="499" uniqueCount="249">
   <si>
     <t xml:space="preserve">Induplac IoT — Cargos del equipo (Nota 2, punto 2)</t>
   </si>
   <si>
-    <t xml:space="preserve">Autora: Bárbara Saavedra · actualizado 19/10/2026 · Las celdas amarillas las completa cada integrante.</t>
+    <t xml:space="preserve">Autora: Bárbara Saavedra · actualizado 21/10/2026 · Las celdas amarillas las completa cada integrante.</t>
   </si>
   <si>
     <t xml:space="preserve">Integrante</t>
@@ -86,6 +64,9 @@
     <t xml:space="preserve">Todos (transversal)</t>
   </si>
   <si>
+    <t xml:space="preserve">Redes e integración de sistemas: diseña la arquitectura completa (red, broker, Edge y nube) y coordina el repositorio y el trabajo del equipo.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Sebastián Fuentes</t>
   </si>
   <si>
@@ -101,6 +82,9 @@
     <t xml:space="preserve">Sprint 2 y 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Electrónica y prototipado IoT: arma el circuito y el firmware del ESP32 (sensores, MQTT con TLS, buffer offline) y resuelve problemas de hardware simulado.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Lisandra González</t>
   </si>
   <si>
@@ -116,6 +100,9 @@
     <t xml:space="preserve">Sprint 3</t>
   </si>
   <si>
+    <t xml:space="preserve">Pendiente (se define con ella).</t>
+  </si>
+  <si>
     <t xml:space="preserve">Felipe Murúa</t>
   </si>
   <si>
@@ -128,6 +115,9 @@
     <t xml:space="preserve">backend/, infrastructure/</t>
   </si>
   <si>
+    <t xml:space="preserve">Cloud y seguridad en AWS: configura y administra los servicios (Lambda, RDS, Cognito con MFA, security groups) cuidando el costo y el acceso mínimo.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Bárbara Saavedra</t>
   </si>
   <si>
@@ -143,6 +133,9 @@
     <t xml:space="preserve">Sprint 3 e implementación</t>
   </si>
   <si>
+    <t xml:space="preserve">Planificación y documentación: organiza el proyecto con RACI, Carta Gantt, Scrum y PMI, y traduce lo técnico a documentos claros.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Roles Scrum (MVP)</t>
   </si>
   <si>
@@ -209,24 +202,45 @@
     <t xml:space="preserve">Dashboard React con datos simulados y conexión a la API</t>
   </si>
   <si>
+    <t xml:space="preserve">Listo (PR #18)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Edge Gateway en Python: SQLite, intervalos de 15 min, alertas y sincronización</t>
   </si>
   <si>
     <t xml:space="preserve">Backend AWS y base RDS junto a Felipe</t>
   </si>
   <si>
+    <t xml:space="preserve">Listo (PR #16)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Login del dashboard con Cognito y MFA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">En curso (PR #20, falta probar con Felipe)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pipeline DevOps: GitHub Actions (CI en cada PR y despliegue a AWS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listo (PR #21)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Casos de prueba y ensayo de la demo</t>
   </si>
   <si>
+    <t xml:space="preserve">Sebastián</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sketch ESP32 en Wokwi: Local 1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sketch ESP32 en Wokwi: Local 2</t>
+  </si>
+  <si>
     <t xml:space="preserve">Pendiente</t>
   </si>
   <si>
-    <t xml:space="preserve">Sebastián</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sketch ESP32 en Wokwi (Local 1 y Local 2)</t>
-  </si>
-  <si>
     <t xml:space="preserve">Sensores simulados: CT (kW), caudalímetro (agua) y UV</t>
   </si>
   <si>
@@ -275,13 +289,19 @@
     <t xml:space="preserve">Dashboard publicado en S3</t>
   </si>
   <si>
-    <t xml:space="preserve">RDS PostgreSQL: permisos, umbrales y catálogo (se enciende para la demo)</t>
+    <t xml:space="preserve">RDS PostgreSQL: permisos, umbrales y catálogo + Lambda induplac-config</t>
   </si>
   <si>
     <t xml:space="preserve">Re-deploy de la Lambda con alertas del Edge</t>
   </si>
   <si>
-    <t xml:space="preserve">Cognito con MFA</t>
+    <t xml:space="preserve">Listo (20/10)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cognito con MFA (user pool, clave temporal y MFA TOTP)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listo: probado en AWS</t>
   </si>
   <si>
     <t xml:space="preserve">IAM, TLS, clave de ingesta y cumplimiento Ley 19.628</t>
@@ -321,6 +341,12 @@
   </si>
   <si>
     <t xml:space="preserve">Listo (PR #14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Actualización de la Nota 2 con lo construido el 20/10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Listo (PR #25)</t>
   </si>
   <si>
     <t xml:space="preserve">Capacitación de usuarios del dashboard</t>
@@ -394,7 +420,7 @@
     <t xml:space="preserve">R</t>
   </si>
   <si>
-    <t xml:space="preserve">Backend AWS: API Gateway, Lambda, DynamoDB, RDS PostgreSQL, S3 y reglas de alerta</t>
+    <t xml:space="preserve">Backend AWS: API Gateway, Lambdas (ingesta e induplac-config), DynamoDB, RDS PostgreSQL, S3 y reglas de alerta</t>
   </si>
   <si>
     <t xml:space="preserve">Dashboard React (vistas por sede, alertas, histórico, panel de demo)</t>
@@ -412,7 +438,7 @@
     <t xml:space="preserve">A</t>
   </si>
   <si>
-    <t xml:space="preserve">Documentación, Pull Requests, demo y presentación final</t>
+    <t xml:space="preserve">Documentación, Pull Requests, pipeline DevOps (GitHub Actions), demo y presentación final</t>
   </si>
   <si>
     <t xml:space="preserve">Actividades como R (incluye A/R)</t>
@@ -430,7 +456,7 @@
     <t xml:space="preserve">Inicio del proyecto (lunes semana 1):</t>
   </si>
   <si>
-    <t xml:space="preserve">Cambia esta fecha o las de Inicio/Duración (azul) y todo se recalcula. ■ = semana de trabajo · ◆ = hito</t>
+    <t xml:space="preserve">Cambia esta fecha o las de Inicio/Duración (azul) y todo se recalcula. ■ = semana de trabajo · ◆ = hito · actualizado 21/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">ID</t>
@@ -535,7 +561,7 @@
     <t xml:space="preserve">2.3</t>
   </si>
   <si>
-    <t xml:space="preserve">Dashboard React con datos simulados</t>
+    <t xml:space="preserve">Dashboard React (datos simulados y API de AWS)</t>
   </si>
   <si>
     <t xml:space="preserve">2.4</t>
@@ -544,6 +570,9 @@
     <t xml:space="preserve">Backend AWS: API Gateway, Lambda, DynamoDB y S3</t>
   </si>
   <si>
+    <t xml:space="preserve">Felipe y Abraham</t>
+  </si>
+  <si>
     <t xml:space="preserve">3</t>
   </si>
   <si>
@@ -553,7 +582,7 @@
     <t xml:space="preserve">3.1</t>
   </si>
   <si>
-    <t xml:space="preserve">ESP32 en Wokwi publicando por MQTT</t>
+    <t xml:space="preserve">ESP32 en Wokwi publicando por MQTT (Local 1 listo; Local 2 pendiente)</t>
   </si>
   <si>
     <t xml:space="preserve">3.2</t>
@@ -571,6 +600,9 @@
     <t xml:space="preserve">3.4</t>
   </si>
   <si>
+    <t xml:space="preserve">Cognito con MFA (probado en AWS; login del dashboard en PR #20)</t>
+  </si>
+  <si>
     <t xml:space="preserve">2.4, 3.3</t>
   </si>
   <si>
@@ -586,6 +618,12 @@
     <t xml:space="preserve">3.1, 3.2, 3.3</t>
   </si>
   <si>
+    <t xml:space="preserve">3.7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2.3, 3.2</t>
+  </si>
+  <si>
     <t xml:space="preserve">4</t>
   </si>
   <si>
@@ -601,6 +639,9 @@
     <t xml:space="preserve">Inicio: validar alcance y criterios de éxito con Induplac</t>
   </si>
   <si>
+    <t xml:space="preserve">Planificado</t>
+  </si>
+  <si>
     <t xml:space="preserve">4.2</t>
   </si>
   <si>
@@ -688,37 +729,52 @@
     <t xml:space="preserve">Hito</t>
   </si>
   <si>
+    <t xml:space="preserve">Cumplido</t>
+  </si>
+  <si>
     <t xml:space="preserve">5.2</t>
   </si>
   <si>
+    <t xml:space="preserve">◆ MVP funcionando de punta a punta (Wokwi → EMQX → Edge → AWS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.3</t>
+  </si>
+  <si>
     <t xml:space="preserve">◆ Demostración del prototipo (miércoles 21/10)</t>
   </si>
   <si>
-    <t xml:space="preserve">5.3</t>
+    <t xml:space="preserve">Hoy</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.4</t>
   </si>
   <si>
     <t xml:space="preserve">◆ Acta de inicio con Induplac</t>
   </si>
   <si>
-    <t xml:space="preserve">5.4</t>
+    <t xml:space="preserve">5.5</t>
   </si>
   <si>
     <t xml:space="preserve">◆ Pruebas aprobadas</t>
   </si>
   <si>
-    <t xml:space="preserve">5.5</t>
+    <t xml:space="preserve">5.6</t>
   </si>
   <si>
     <t xml:space="preserve">◆ Puesta en marcha</t>
   </si>
   <si>
-    <t xml:space="preserve">Colores por responsable:</t>
+    <t xml:space="preserve">Colores por responsable (si hay dos, manda el primero):</t>
   </si>
   <si>
     <t xml:space="preserve">Lógica PMI: S1–S3 es el desarrollo del MVP con Scrum (ya en ejecución). S4–S12 es la implementación en Induplac con las 5 fases PMI: inicio (S4), planificación (S5), ejecución (S6–S10), monitoreo y control (transversal) y cierre (S12).</t>
   </si>
   <si>
-    <t xml:space="preserve">Cambio 19/10/2026: RDS PostgreSQL vuelve al MVP (tarea 3.3); se mantiene apagado y se enciende para la demo del miércoles y para configuraciones.</t>
+    <t xml:space="preserve">Estado: Listo / Cumplido = terminado · En curso / Hoy = en desarrollo · Pendiente = atrasado o sin empezar · Planificado = implementación futura.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cambios 19/10: RDS PostgreSQL vuelve al MVP (3.3). Cambios 21/10: columna Estado, tarea 3.7 Pipeline DevOps, hito 5.2 MVP de punta a punta (20/10) y responsables compartidos Felipe y Abraham en 2.4, 3.3 y 3.4.</t>
   </si>
 </sst>
 </file>
@@ -730,7 +786,7 @@
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="dd/mm"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -794,11 +850,6 @@
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="2"/>
     </font>
     <font>
       <b val="true"/>
@@ -976,39 +1027,39 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1016,11 +1067,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1028,19 +1079,19 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="166" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1056,31 +1107,31 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="5" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="6" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="8" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="10" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1488,7 +1539,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>8</v>
       </c>
@@ -1504,114 +1555,104 @@
       <c r="E5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="5" t="inlineStr">
-        <is>
-          <t>Redes e integración de sistemas: diseña la arquitectura completa (red, broker, Edge y nube) y coordina el repositorio y el trabajo del equipo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F5" s="5" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="5" t="inlineStr">
-        <is>
-          <t>Electrónica y prototipado IoT: arma el circuito y el firmware del ESP32 (sensores, MQTT con TLS, buffer offline) y resuelve problemas de hardware simulado.</t>
-        </is>
+        <v>18</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="E8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="B7" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F7" s="5" t="inlineStr">
-        <is>
-          <t>Pendiente (se define con ella el 21/10).</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="C8" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="F8" s="5" t="inlineStr">
-        <is>
-          <t>Cloud y seguridad en AWS: configura y administra los servicios (Lambda, RDS, Cognito con MFA, security groups) cuidando el costo y el acceso mínimo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F8" s="5" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
-        <is>
-          <t>Planificación y documentación: organiza el proyecto con RACI, Carta Gantt, Scrum y PMI, y traduce lo técnico a documentos claros.</t>
-        </is>
+        <v>35</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="6" t="s">
-        <v>32</v>
+      <c r="A11" s="7" t="s">
+        <v>37</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>2</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>34</v>
+        <v>39</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
@@ -1619,39 +1660,35 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>Abraham Castro</t>
-        </is>
+        <v>40</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>8</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>36</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="7" t="inlineStr">
-        <is>
-          <t>Bárbara Saavedra</t>
-        </is>
+        <v>42</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>31</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>38</v>
+        <v>43</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>
@@ -1662,7 +1699,6 @@
     <oddHeader/>
     <oddFooter/>
   </headerFooter>
-  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1671,7 +1707,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:D41"/>
+  <dimension ref="A1:D45"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
@@ -1682,7 +1718,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1690,570 +1726,602 @@
         <v>2</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #18)</t>
-        </is>
+        <v>18</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #18)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>18</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="8" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>56</v>
+        <v>63</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D9" s="4" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="9" t="s">
-        <v>58</v>
+      <c r="A10" s="8" t="s">
+        <v>51</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D10" s="4" t="inlineStr">
-        <is>
-          <t>Listo Local 1 (PR #16)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="9" t="s">
-        <v>58</v>
+      <c r="A11" s="8" t="s">
+        <v>51</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>60</v>
+        <v>67</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="9" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>61</v>
+        <v>69</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
+        <v>18</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="9" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>62</v>
+        <v>70</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="9" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D14" s="4" t="inlineStr">
-        <is>
-          <t>En curso</t>
-        </is>
+        <v>24</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="10" t="s">
-        <v>64</v>
+      <c r="A15" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>65</v>
+        <v>73</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="s">
-        <v>64</v>
+      <c r="A16" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="s">
-        <v>64</v>
+      <c r="A17" s="9" t="s">
+        <v>68</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="10" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>68</v>
+        <v>77</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>57</v>
+        <v>71</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11" t="s">
-        <v>70</v>
+      <c r="A19" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B19" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="C19" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="4" t="s">
-        <v>72</v>
-      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11" t="s">
-        <v>70</v>
+      <c r="A20" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>51</v>
+        <v>24</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>70</v>
+      <c r="A21" s="10" t="s">
+        <v>76</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>51</v>
+        <v>81</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>72</v>
+        <v>84</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>76</v>
+        <v>85</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D23" s="4" t="inlineStr">
-        <is>
-          <t>Listo (PR #16)</t>
-        </is>
+        <v>56</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>77</v>
+        <v>86</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D24" s="4" t="inlineStr">
-        <is>
-          <t>Listo (20/10)</t>
-        </is>
+        <v>56</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>78</v>
+        <v>87</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D25" s="4" t="inlineStr">
-        <is>
-          <t>Listo: probado en AWS (falta conectarlo al dashboard)</t>
-        </is>
+        <v>56</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>84</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>79</v>
+        <v>88</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>49</v>
+        <v>62</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
-        <v>80</v>
+      <c r="A27" s="11" t="s">
+        <v>82</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D27" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
-        <v>80</v>
-      </c>
       <c r="B28" s="4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D28" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
-        <v>80</v>
-      </c>
       <c r="B29" s="4" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>85</v>
+        <v>54</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>86</v>
+        <v>95</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="12" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>69</v>
+        <v>24</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>57</v>
+        <v>101</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B34" s="4" t="s">
+        <v>102</v>
+      </c>
+      <c r="C34" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D34" s="4" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="13" t="s">
-        <v>93</v>
+      <c r="A35" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B35" s="4" t="s">
+        <v>104</v>
+      </c>
+      <c r="C35" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D35" s="4" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="3" t="s">
+      <c r="A36" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>106</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D36" s="4" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="B37" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="C37" s="4" t="s">
+        <v>81</v>
+      </c>
+      <c r="D37" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B36" s="3" t="s">
-        <v>94</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B37" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A37)</f>
-        <v>6</v>
-      </c>
-      <c r="C37" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A37,$D$4:$D$33,"Listo*")</f>
-        <v>1</v>
-      </c>
-      <c r="D37" s="14" t="n">
-        <f aca="false">B37-C37</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="14" t="s">
-        <v>58</v>
-      </c>
-      <c r="B38" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A38)</f>
-        <v>5</v>
-      </c>
-      <c r="C38" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A38,$D$4:$D$33,"Listo*")</f>
-        <v>0</v>
-      </c>
-      <c r="D38" s="14" t="n">
-        <f aca="false">B38-C38</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="B39" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A39)</f>
-        <v>4</v>
-      </c>
-      <c r="C39" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A39,$D$4:$D$33,"Listo*")</f>
-        <v>0</v>
-      </c>
-      <c r="D39" s="14" t="n">
-        <f aca="false">B39-C39</f>
-        <v>4</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="14" t="s">
-        <v>70</v>
-      </c>
-      <c r="B40" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A40)</f>
-        <v>8</v>
-      </c>
-      <c r="C40" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A40,$D$4:$D$33,"Listo*")</f>
-        <v>4</v>
-      </c>
-      <c r="D40" s="14" t="n">
-        <f aca="false">B40-C40</f>
-        <v>4</v>
+      <c r="B40" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D40" s="3" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="14" t="s">
-        <v>80</v>
+        <v>51</v>
       </c>
       <c r="B41" s="14" t="n">
-        <f aca="false">COUNTIF($A$4:$A$33,A41)</f>
-        <v>7</v>
+        <f aca="false">COUNTIF($A$4:$A$37,A41)</f>
+        <v>8</v>
       </c>
       <c r="C41" s="14" t="n">
-        <f aca="false">COUNTIFS($A$4:$A$33,A41,$D$4:$D$33,"Listo*")</f>
-        <v>6</v>
+        <f aca="false">COUNTIFS($A$4:$A$37,A41,$D$4:$D$37,"Listo*")</f>
+        <v>5</v>
       </c>
       <c r="D41" s="14" t="n">
         <f aca="false">B41-C41</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="14" t="s">
+        <v>68</v>
+      </c>
+      <c r="B42" s="14" t="n">
+        <f aca="false">COUNTIF($A$4:$A$37,A42)</f>
+        <v>6</v>
+      </c>
+      <c r="C42" s="14" t="n">
+        <f aca="false">COUNTIFS($A$4:$A$37,A42,$D$4:$D$37,"Listo*")</f>
+        <v>4</v>
+      </c>
+      <c r="D42" s="14" t="n">
+        <f aca="false">B42-C42</f>
+        <v>2</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="14" t="s">
+        <v>76</v>
+      </c>
+      <c r="B43" s="14" t="n">
+        <f aca="false">COUNTIF($A$4:$A$37,A43)</f>
+        <v>4</v>
+      </c>
+      <c r="C43" s="14" t="n">
+        <f aca="false">COUNTIFS($A$4:$A$37,A43,$D$4:$D$37,"Listo*")</f>
+        <v>0</v>
+      </c>
+      <c r="D43" s="14" t="n">
+        <f aca="false">B43-C43</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="14" t="s">
+        <v>82</v>
+      </c>
+      <c r="B44" s="14" t="n">
+        <f aca="false">COUNTIF($A$4:$A$37,A44)</f>
+        <v>8</v>
+      </c>
+      <c r="C44" s="14" t="n">
+        <f aca="false">COUNTIFS($A$4:$A$37,A44,$D$4:$D$37,"Listo*")</f>
+        <v>7</v>
+      </c>
+      <c r="D44" s="14" t="n">
+        <f aca="false">B44-C44</f>
         <v>1</v>
       </c>
     </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="14" t="s">
+        <v>94</v>
+      </c>
+      <c r="B45" s="14" t="n">
+        <f aca="false">COUNTIF($A$4:$A$37,A45)</f>
+        <v>8</v>
+      </c>
+      <c r="C45" s="14" t="n">
+        <f aca="false">COUNTIFS($A$4:$A$37,A45,$D$4:$D$37,"Listo*")</f>
+        <v>7</v>
+      </c>
+      <c r="D45" s="14" t="n">
+        <f aca="false">B45-C45</f>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="D4:D33">
+  <conditionalFormatting sqref="D4:D37">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
       <formula>LEFT(D4,5)="Listo"</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
-      <formula>D4="En curso"</formula>
+      <formula>LEFT(D4,8)="En curso"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -2282,38 +2350,38 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>97</v>
+        <v>113</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>98</v>
+        <v>114</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>99</v>
+        <v>115</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>100</v>
+        <v>116</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>101</v>
+        <v>117</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>102</v>
+        <v>118</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>103</v>
+        <v>119</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>104</v>
+        <v>120</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>105</v>
+        <v>121</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>106</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2321,22 +2389,22 @@
         <v>1</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>107</v>
+        <v>123</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H5" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C5:G5,"*R*")&gt;=1,COUNTIF(C5:G5,"A*")=1),"OK","Revisar")</f>
@@ -2348,22 +2416,22 @@
         <v>2</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D6" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="E6" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="F6" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G6" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H6" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C6:G6,"*R*")&gt;=1,COUNTIF(C6:G6,"A*")=1),"OK","Revisar")</f>
@@ -2375,22 +2443,22 @@
         <v>3</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>111</v>
+        <v>127</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H7" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C7:G7,"*R*")&gt;=1,COUNTIF(C7:G7,"A*")=1),"OK","Revisar")</f>
@@ -2402,22 +2470,22 @@
         <v>4</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>112</v>
+        <v>128</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H8" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C8:G8,"*R*")&gt;=1,COUNTIF(C8:G8,"A*")=1),"OK","Revisar")</f>
@@ -2429,22 +2497,22 @@
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>114</v>
+        <v>130</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E9" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="F9" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H9" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C9:G9,"*R*")&gt;=1,COUNTIF(C9:G9,"A*")=1),"OK","Revisar")</f>
@@ -2456,22 +2524,22 @@
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>115</v>
+        <v>131</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D10" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E10" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="F10" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G10" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="H10" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C10:G10,"*R*")&gt;=1,COUNTIF(C10:G10,"A*")=1),"OK","Revisar")</f>
@@ -2483,22 +2551,22 @@
         <v>7</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>116</v>
+        <v>132</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D11" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="E11" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="F11" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="G11" s="15" t="s">
-        <v>110</v>
+        <v>126</v>
       </c>
       <c r="H11" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C11:G11,"*R*")&gt;=1,COUNTIF(C11:G11,"A*")=1),"OK","Revisar")</f>
@@ -2510,22 +2578,22 @@
         <v>8</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>117</v>
+        <v>133</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="D12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="E12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="F12" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G12" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="H12" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C12:G12,"*R*")&gt;=1,COUNTIF(C12:G12,"A*")=1),"OK","Revisar")</f>
@@ -2537,49 +2605,49 @@
         <v>9</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>118</v>
+        <v>134</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>119</v>
+        <v>135</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>108</v>
+        <v>124</v>
       </c>
       <c r="H13" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C13:G13,"*R*")&gt;=1,COUNTIF(C13:G13,"A*")=1),"OK","Revisar")</f>
         <v>OK</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="n">
         <v>10</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>120</v>
+        <v>136</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="D14" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="E14" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="F14" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="G14" s="15" t="s">
-        <v>113</v>
+        <v>129</v>
       </c>
       <c r="H14" s="14" t="str">
         <f aca="false">IF(AND(COUNTIF(C14:G14,"*R*")&gt;=1,COUNTIF(C14:G14,"A*")=1),"OK","Revisar")</f>
@@ -2588,7 +2656,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="16" t="s">
-        <v>121</v>
+        <v>137</v>
       </c>
       <c r="C16" s="14" t="n">
         <f aca="false">COUNTIF(C5:C14,"*R*")</f>
@@ -2613,7 +2681,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="16" t="s">
-        <v>122</v>
+        <v>138</v>
       </c>
       <c r="C17" s="14" t="n">
         <f aca="false">COUNTIF(C5:C14,"A*")</f>
@@ -2638,7 +2706,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="2" t="s">
-        <v>123</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -2665,161 +2733,164 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:T48"/>
+  <dimension ref="A1:U51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="6"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="9"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="20" min="9" style="0" width="6"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="21" min="10" style="0" width="6"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>140</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="E2" s="18" t="n">
         <v>46300</v>
       </c>
-      <c r="F2" s="2" t="s">
-        <v>126</v>
+      <c r="G2" s="2" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>127</v>
+        <v>143</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>129</v>
+        <v>145</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>130</v>
+        <v>146</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>131</v>
+        <v>147</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>132</v>
+        <v>148</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>133</v>
+        <v>149</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>134</v>
+        <v>50</v>
       </c>
       <c r="J4" s="3" t="s">
-        <v>135</v>
+        <v>150</v>
       </c>
       <c r="K4" s="3" t="s">
-        <v>136</v>
+        <v>151</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>137</v>
+        <v>152</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>138</v>
+        <v>153</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>139</v>
+        <v>154</v>
       </c>
       <c r="O4" s="3" t="s">
-        <v>140</v>
+        <v>155</v>
       </c>
       <c r="P4" s="3" t="s">
-        <v>141</v>
+        <v>156</v>
       </c>
       <c r="Q4" s="3" t="s">
-        <v>142</v>
+        <v>157</v>
       </c>
       <c r="R4" s="3" t="s">
-        <v>143</v>
+        <v>158</v>
       </c>
       <c r="S4" s="3" t="s">
-        <v>144</v>
+        <v>159</v>
       </c>
       <c r="T4" s="3" t="s">
-        <v>145</v>
+        <v>160</v>
+      </c>
+      <c r="U4" s="3" t="s">
+        <v>161</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B5" s="19" t="s">
-        <v>146</v>
-      </c>
-      <c r="I5" s="20" t="n">
+        <v>162</v>
+      </c>
+      <c r="J5" s="20" t="n">
         <f aca="false">$E$2+0</f>
         <v>46300</v>
       </c>
-      <c r="J5" s="20" t="n">
+      <c r="K5" s="20" t="n">
         <f aca="false">$E$2+7</f>
         <v>46307</v>
       </c>
-      <c r="K5" s="20" t="n">
+      <c r="L5" s="20" t="n">
         <f aca="false">$E$2+14</f>
         <v>46314</v>
       </c>
-      <c r="L5" s="20" t="n">
+      <c r="M5" s="20" t="n">
         <f aca="false">$E$2+21</f>
         <v>46321</v>
       </c>
-      <c r="M5" s="20" t="n">
+      <c r="N5" s="20" t="n">
         <f aca="false">$E$2+28</f>
         <v>46328</v>
       </c>
-      <c r="N5" s="20" t="n">
+      <c r="O5" s="20" t="n">
         <f aca="false">$E$2+35</f>
         <v>46335</v>
       </c>
-      <c r="O5" s="20" t="n">
+      <c r="P5" s="20" t="n">
         <f aca="false">$E$2+42</f>
         <v>46342</v>
       </c>
-      <c r="P5" s="20" t="n">
+      <c r="Q5" s="20" t="n">
         <f aca="false">$E$2+49</f>
         <v>46349</v>
       </c>
-      <c r="Q5" s="20" t="n">
+      <c r="R5" s="20" t="n">
         <f aca="false">$E$2+56</f>
         <v>46356</v>
       </c>
-      <c r="R5" s="20" t="n">
+      <c r="S5" s="20" t="n">
         <f aca="false">$E$2+63</f>
         <v>46363</v>
       </c>
-      <c r="S5" s="20" t="n">
+      <c r="T5" s="20" t="n">
         <f aca="false">$E$2+70</f>
         <v>46370</v>
       </c>
-      <c r="T5" s="20" t="n">
+      <c r="U5" s="20" t="n">
         <f aca="false">$E$2+77</f>
         <v>46377</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="21" t="s">
-        <v>147</v>
+        <v>163</v>
       </c>
       <c r="B6" s="21" t="s">
-        <v>148</v>
+        <v>164</v>
       </c>
       <c r="C6" s="21"/>
       <c r="D6" s="21" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="E6" s="21"/>
       <c r="F6" s="21"/>
@@ -2837,19 +2908,20 @@
       <c r="R6" s="21"/>
       <c r="S6" s="21"/>
       <c r="T6" s="21"/>
+      <c r="U6" s="21"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>150</v>
+        <v>166</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>151</v>
+        <v>167</v>
       </c>
       <c r="C7" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>149</v>
+        <v>165</v>
       </c>
       <c r="E7" s="22" t="n">
         <v>46300</v>
@@ -2862,15 +2934,14 @@
         <v>46304</v>
       </c>
       <c r="H7" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="I7" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E7-6,I$5&lt;=$G7),"■","")</f>
-        <v>■</v>
+        <v>168</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J7" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E7-6,J$5&lt;=$G7),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="K7" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E7-6,K$5&lt;=$G7),"■","")</f>
@@ -2912,19 +2983,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E7-6,T$5&lt;=$G7),"■","")</f>
         <v/>
       </c>
+      <c r="U7" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E7-6,U$5&lt;=$G7),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="8" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>153</v>
+        <v>169</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>154</v>
+        <v>170</v>
       </c>
       <c r="C8" s="14" t="s">
-        <v>80</v>
+        <v>94</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E8" s="22" t="n">
         <v>46307</v>
@@ -2937,15 +3012,14 @@
         <v>46318</v>
       </c>
       <c r="H8" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="I8" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E8-6,I$5&lt;=$G8),"■","")</f>
-        <v/>
+        <v>166</v>
+      </c>
+      <c r="I8" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J8" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E8-6,J$5&lt;=$G8),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K8" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E8-6,K$5&lt;=$G8),"■","")</f>
@@ -2953,7 +3027,7 @@
       </c>
       <c r="L8" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E8-6,L$5&lt;=$G8),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M8" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E8-6,M$5&lt;=$G8),"■","")</f>
@@ -2987,17 +3061,21 @@
         <f aca="false">IF(AND(T$5&gt;=$E8-6,T$5&lt;=$G8),"■","")</f>
         <v/>
       </c>
+      <c r="U8" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E8-6,U$5&lt;=$G8),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="21" t="s">
-        <v>155</v>
+        <v>171</v>
       </c>
       <c r="B9" s="21" t="s">
-        <v>156</v>
+        <v>172</v>
       </c>
       <c r="C9" s="21"/>
       <c r="D9" s="21" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E9" s="21"/>
       <c r="F9" s="21"/>
@@ -3015,19 +3093,20 @@
       <c r="R9" s="21"/>
       <c r="S9" s="21"/>
       <c r="T9" s="21"/>
+      <c r="U9" s="21"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>157</v>
+        <v>173</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>158</v>
+        <v>174</v>
       </c>
       <c r="C10" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E10" s="22" t="n">
         <v>46307</v>
@@ -3040,19 +3119,18 @@
         <v>46311</v>
       </c>
       <c r="H10" s="14" t="s">
-        <v>150</v>
-      </c>
-      <c r="I10" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E10-6,I$5&lt;=$G10),"■","")</f>
-        <v/>
+        <v>166</v>
+      </c>
+      <c r="I10" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J10" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E10-6,J$5&lt;=$G10),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K10" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E10-6,K$5&lt;=$G10),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L10" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E10-6,L$5&lt;=$G10),"■","")</f>
@@ -3090,19 +3168,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E10-6,T$5&lt;=$G10),"■","")</f>
         <v/>
       </c>
+      <c r="U10" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E10-6,U$5&lt;=$G10),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>159</v>
+        <v>175</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C11" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="E11" s="22" t="n">
         <v>46307</v>
@@ -3115,19 +3197,18 @@
         <v>46311</v>
       </c>
       <c r="H11" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="I11" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E11-6,I$5&lt;=$G11),"■","")</f>
-        <v/>
+        <v>173</v>
+      </c>
+      <c r="I11" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J11" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E11-6,J$5&lt;=$G11),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K11" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E11-6,K$5&lt;=$G11),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="L11" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E11-6,L$5&lt;=$G11),"■","")</f>
@@ -3165,19 +3246,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E11-6,T$5&lt;=$G11),"■","")</f>
         <v/>
       </c>
+      <c r="U11" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E11-6,U$5&lt;=$G11),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>160</v>
+        <v>176</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>161</v>
+        <v>177</v>
       </c>
       <c r="C12" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E12" s="22" t="n">
         <v>46307</v>
@@ -3190,15 +3275,14 @@
         <v>46318</v>
       </c>
       <c r="H12" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="I12" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E12-6,I$5&lt;=$G12),"■","")</f>
-        <v/>
+        <v>173</v>
+      </c>
+      <c r="I12" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J12" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E12-6,J$5&lt;=$G12),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K12" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E12-6,K$5&lt;=$G12),"■","")</f>
@@ -3206,7 +3290,7 @@
       </c>
       <c r="L12" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E12-6,L$5&lt;=$G12),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M12" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E12-6,M$5&lt;=$G12),"■","")</f>
@@ -3240,19 +3324,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E12-6,T$5&lt;=$G12),"■","")</f>
         <v/>
       </c>
+      <c r="U12" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E12-6,U$5&lt;=$G12),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="14" t="s">
-        <v>162</v>
+        <v>178</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>163</v>
+        <v>179</v>
       </c>
       <c r="C13" s="14" t="s">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E13" s="22" t="n">
         <v>46307</v>
@@ -3265,15 +3353,14 @@
         <v>46318</v>
       </c>
       <c r="H13" s="14" t="s">
-        <v>157</v>
-      </c>
-      <c r="I13" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E13-6,I$5&lt;=$G13),"■","")</f>
-        <v/>
+        <v>173</v>
+      </c>
+      <c r="I13" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J13" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E13-6,J$5&lt;=$G13),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K13" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E13-6,K$5&lt;=$G13),"■","")</f>
@@ -3281,7 +3368,7 @@
       </c>
       <c r="L13" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E13-6,L$5&lt;=$G13),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M13" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E13-6,M$5&lt;=$G13),"■","")</f>
@@ -3315,17 +3402,21 @@
         <f aca="false">IF(AND(T$5&gt;=$E13-6,T$5&lt;=$G13),"■","")</f>
         <v/>
       </c>
+      <c r="U13" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E13-6,U$5&lt;=$G13),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="21" t="s">
-        <v>164</v>
+        <v>181</v>
       </c>
       <c r="B14" s="21" t="s">
-        <v>165</v>
+        <v>182</v>
       </c>
       <c r="C14" s="21"/>
       <c r="D14" s="21" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E14" s="21"/>
       <c r="F14" s="21"/>
@@ -3343,19 +3434,20 @@
       <c r="R14" s="21"/>
       <c r="S14" s="21"/>
       <c r="T14" s="21"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U14" s="21"/>
+    </row>
+    <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>166</v>
+        <v>183</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="C15" s="14" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E15" s="22" t="n">
         <v>46307</v>
@@ -3368,15 +3460,14 @@
         <v>46318</v>
       </c>
       <c r="H15" s="14" t="s">
-        <v>159</v>
-      </c>
-      <c r="I15" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E15-6,I$5&lt;=$G15),"■","")</f>
-        <v/>
+        <v>175</v>
+      </c>
+      <c r="I15" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="J15" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E15-6,J$5&lt;=$G15),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K15" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E15-6,K$5&lt;=$G15),"■","")</f>
@@ -3384,7 +3475,7 @@
       </c>
       <c r="L15" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E15-6,L$5&lt;=$G15),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M15" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E15-6,M$5&lt;=$G15),"■","")</f>
@@ -3418,19 +3509,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E15-6,T$5&lt;=$G15),"■","")</f>
         <v/>
       </c>
+      <c r="U15" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E15-6,U$5&lt;=$G15),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>168</v>
+        <v>185</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>169</v>
+        <v>186</v>
       </c>
       <c r="C16" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E16" s="22" t="n">
         <v>46307</v>
@@ -3443,15 +3538,14 @@
         <v>46318</v>
       </c>
       <c r="H16" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="I16" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E16-6,I$5&lt;=$G16),"■","")</f>
-        <v/>
+        <v>187</v>
+      </c>
+      <c r="I16" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J16" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E16-6,J$5&lt;=$G16),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="K16" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E16-6,K$5&lt;=$G16),"■","")</f>
@@ -3459,7 +3553,7 @@
       </c>
       <c r="L16" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E16-6,L$5&lt;=$G16),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M16" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E16-6,M$5&lt;=$G16),"■","")</f>
@@ -3493,19 +3587,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E16-6,T$5&lt;=$G16),"■","")</f>
         <v/>
       </c>
+      <c r="U16" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E16-6,U$5&lt;=$G16),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="14" t="s">
-        <v>171</v>
+        <v>188</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>76</v>
+        <v>88</v>
       </c>
       <c r="C17" s="14" t="s">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E17" s="22" t="n">
         <v>46314</v>
@@ -3518,11 +3616,10 @@
         <v>46318</v>
       </c>
       <c r="H17" s="14" t="s">
-        <v>162</v>
-      </c>
-      <c r="I17" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E17-6,I$5&lt;=$G17),"■","")</f>
-        <v/>
+        <v>178</v>
+      </c>
+      <c r="I17" s="14" t="s">
+        <v>84</v>
       </c>
       <c r="J17" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E17-6,J$5&lt;=$G17),"■","")</f>
@@ -3530,11 +3627,11 @@
       </c>
       <c r="K17" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E17-6,K$5&lt;=$G17),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="L17" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E17-6,L$5&lt;=$G17),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M17" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E17-6,M$5&lt;=$G17),"■","")</f>
@@ -3568,19 +3665,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E17-6,T$5&lt;=$G17),"■","")</f>
         <v/>
       </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U17" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E17-6,U$5&lt;=$G17),"■","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="s">
-        <v>172</v>
+        <v>189</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>78</v>
+        <v>190</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>70</v>
+        <v>180</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E18" s="22" t="n">
         <v>46314</v>
@@ -3593,11 +3694,10 @@
         <v>46318</v>
       </c>
       <c r="H18" s="14" t="s">
-        <v>173</v>
-      </c>
-      <c r="I18" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E18-6,I$5&lt;=$G18),"■","")</f>
-        <v/>
+        <v>191</v>
+      </c>
+      <c r="I18" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="J18" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E18-6,J$5&lt;=$G18),"■","")</f>
@@ -3605,11 +3705,11 @@
       </c>
       <c r="K18" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E18-6,K$5&lt;=$G18),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="L18" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E18-6,L$5&lt;=$G18),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M18" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E18-6,M$5&lt;=$G18),"■","")</f>
@@ -3643,19 +3743,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E18-6,T$5&lt;=$G18),"■","")</f>
         <v/>
       </c>
+      <c r="U18" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E18-6,U$5&lt;=$G18),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="s">
-        <v>174</v>
+        <v>192</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>175</v>
+        <v>193</v>
       </c>
       <c r="C19" s="14" t="s">
-        <v>64</v>
+        <v>76</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E19" s="22" t="n">
         <v>46314</v>
@@ -3668,11 +3772,10 @@
         <v>46318</v>
       </c>
       <c r="H19" s="14" t="s">
-        <v>168</v>
-      </c>
-      <c r="I19" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E19-6,I$5&lt;=$G19),"■","")</f>
-        <v/>
+        <v>185</v>
+      </c>
+      <c r="I19" s="14" t="s">
+        <v>71</v>
       </c>
       <c r="J19" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E19-6,J$5&lt;=$G19),"■","")</f>
@@ -3680,11 +3783,11 @@
       </c>
       <c r="K19" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E19-6,K$5&lt;=$G19),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="L19" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E19-6,L$5&lt;=$G19),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M19" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E19-6,M$5&lt;=$G19),"■","")</f>
@@ -3718,19 +3821,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E19-6,T$5&lt;=$G19),"■","")</f>
         <v/>
       </c>
+      <c r="U19" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E19-6,U$5&lt;=$G19),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="s">
-        <v>176</v>
+        <v>194</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="C20" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E20" s="22" t="n">
         <v>46314</v>
@@ -3743,11 +3850,10 @@
         <v>46318</v>
       </c>
       <c r="H20" s="14" t="s">
-        <v>177</v>
-      </c>
-      <c r="I20" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E20-6,I$5&lt;=$G20),"■","")</f>
-        <v/>
+        <v>195</v>
+      </c>
+      <c r="I20" s="14" t="s">
+        <v>54</v>
       </c>
       <c r="J20" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E20-6,J$5&lt;=$G20),"■","")</f>
@@ -3755,11 +3861,11 @@
       </c>
       <c r="K20" s="25" t="str">
         <f aca="false">IF(AND(K$5&gt;=$E20-6,K$5&lt;=$G20),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="L20" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E20-6,L$5&lt;=$G20),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="M20" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E20-6,M$5&lt;=$G20),"■","")</f>
@@ -3793,139 +3899,146 @@
         <f aca="false">IF(AND(T$5&gt;=$E20-6,T$5&lt;=$G20),"■","")</f>
         <v/>
       </c>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="s">
-        <v>178</v>
-      </c>
-      <c r="B21" s="21" t="s">
-        <v>179</v>
-      </c>
-      <c r="C21" s="21"/>
-      <c r="D21" s="21" t="s">
-        <v>180</v>
-      </c>
-      <c r="E21" s="21"/>
-      <c r="F21" s="21"/>
-      <c r="G21" s="21"/>
-      <c r="H21" s="21"/>
-      <c r="I21" s="21"/>
-      <c r="J21" s="21"/>
-      <c r="K21" s="21"/>
-      <c r="L21" s="21"/>
-      <c r="M21" s="21"/>
-      <c r="N21" s="21"/>
-      <c r="O21" s="21"/>
-      <c r="P21" s="21"/>
-      <c r="Q21" s="21"/>
-      <c r="R21" s="21"/>
-      <c r="S21" s="21"/>
-      <c r="T21" s="21"/>
+      <c r="U20" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E20-6,U$5&lt;=$G20),"■","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="s">
+        <v>196</v>
+      </c>
+      <c r="B21" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="C21" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D21" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" s="22" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F21" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" s="24" t="n">
+        <f aca="false">E21+F21*7-3</f>
+        <v>46318</v>
+      </c>
+      <c r="H21" s="14" t="s">
+        <v>197</v>
+      </c>
+      <c r="I21" s="14" t="s">
+        <v>84</v>
+      </c>
+      <c r="J21" s="25" t="str">
+        <f aca="false">IF(AND(J$5&gt;=$E21-6,J$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="K21" s="25" t="str">
+        <f aca="false">IF(AND(K$5&gt;=$E21-6,K$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="L21" s="25" t="str">
+        <f aca="false">IF(AND(L$5&gt;=$E21-6,L$5&lt;=$G21),"■","")</f>
+        <v>■</v>
+      </c>
+      <c r="M21" s="25" t="str">
+        <f aca="false">IF(AND(M$5&gt;=$E21-6,M$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="N21" s="25" t="str">
+        <f aca="false">IF(AND(N$5&gt;=$E21-6,N$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="O21" s="25" t="str">
+        <f aca="false">IF(AND(O$5&gt;=$E21-6,O$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="P21" s="25" t="str">
+        <f aca="false">IF(AND(P$5&gt;=$E21-6,P$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="Q21" s="25" t="str">
+        <f aca="false">IF(AND(Q$5&gt;=$E21-6,Q$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="R21" s="25" t="str">
+        <f aca="false">IF(AND(R$5&gt;=$E21-6,R$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="S21" s="25" t="str">
+        <f aca="false">IF(AND(S$5&gt;=$E21-6,S$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="T21" s="25" t="str">
+        <f aca="false">IF(AND(T$5&gt;=$E21-6,T$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
+      <c r="U21" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E21-6,U$5&lt;=$G21),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="B22" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="C22" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="D22" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="E22" s="22" t="n">
+      <c r="A22" s="21" t="s">
+        <v>198</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>199</v>
+      </c>
+      <c r="C22" s="21"/>
+      <c r="D22" s="21" t="s">
+        <v>200</v>
+      </c>
+      <c r="E22" s="21"/>
+      <c r="F22" s="21"/>
+      <c r="G22" s="21"/>
+      <c r="H22" s="21"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="21"/>
+      <c r="K22" s="21"/>
+      <c r="L22" s="21"/>
+      <c r="M22" s="21"/>
+      <c r="N22" s="21"/>
+      <c r="O22" s="21"/>
+      <c r="P22" s="21"/>
+      <c r="Q22" s="21"/>
+      <c r="R22" s="21"/>
+      <c r="S22" s="21"/>
+      <c r="T22" s="21"/>
+      <c r="U22" s="21"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="14" t="s">
+        <v>201</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="C23" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="E23" s="22" t="n">
         <v>46321</v>
-      </c>
-      <c r="F22" s="23" t="n">
-        <v>1</v>
-      </c>
-      <c r="G22" s="24" t="n">
-        <f aca="false">E22+F22*7-3</f>
-        <v>46325</v>
-      </c>
-      <c r="H22" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="I22" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E22-6,I$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="J22" s="25" t="str">
-        <f aca="false">IF(AND(J$5&gt;=$E22-6,J$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="K22" s="25" t="str">
-        <f aca="false">IF(AND(K$5&gt;=$E22-6,K$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="L22" s="25" t="str">
-        <f aca="false">IF(AND(L$5&gt;=$E22-6,L$5&lt;=$G22),"■","")</f>
-        <v>■</v>
-      </c>
-      <c r="M22" s="25" t="str">
-        <f aca="false">IF(AND(M$5&gt;=$E22-6,M$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="N22" s="25" t="str">
-        <f aca="false">IF(AND(N$5&gt;=$E22-6,N$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="O22" s="25" t="str">
-        <f aca="false">IF(AND(O$5&gt;=$E22-6,O$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="P22" s="25" t="str">
-        <f aca="false">IF(AND(P$5&gt;=$E22-6,P$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="Q22" s="25" t="str">
-        <f aca="false">IF(AND(Q$5&gt;=$E22-6,Q$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="R22" s="25" t="str">
-        <f aca="false">IF(AND(R$5&gt;=$E22-6,R$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="S22" s="25" t="str">
-        <f aca="false">IF(AND(S$5&gt;=$E22-6,S$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-      <c r="T22" s="25" t="str">
-        <f aca="false">IF(AND(T$5&gt;=$E22-6,T$5&lt;=$G22),"■","")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="B23" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="C23" s="14" t="s">
-        <v>80</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="E23" s="22" t="n">
-        <v>46328</v>
       </c>
       <c r="F23" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G23" s="24" t="n">
         <f aca="false">E23+F23*7-3</f>
-        <v>46332</v>
+        <v>46325</v>
       </c>
       <c r="H23" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="I23" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E23-6,I$5&lt;=$G23),"■","")</f>
-        <v/>
+        <v>194</v>
+      </c>
+      <c r="I23" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J23" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E23-6,J$5&lt;=$G23),"■","")</f>
@@ -3971,36 +4084,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E23-6,T$5&lt;=$G23),"■","")</f>
         <v/>
       </c>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U23" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E23-6,U$5&lt;=$G23),"■","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="14" t="s">
-        <v>186</v>
+        <v>204</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>187</v>
+        <v>205</v>
       </c>
       <c r="C24" s="14" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>188</v>
+        <v>206</v>
       </c>
       <c r="E24" s="22" t="n">
-        <v>46335</v>
+        <v>46328</v>
       </c>
       <c r="F24" s="23" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G24" s="24" t="n">
         <f aca="false">E24+F24*7-3</f>
-        <v>46346</v>
+        <v>46332</v>
       </c>
       <c r="H24" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="I24" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E24-6,I$5&lt;=$G24),"■","")</f>
-        <v/>
+        <v>201</v>
+      </c>
+      <c r="I24" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J24" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E24-6,J$5&lt;=$G24),"■","")</f>
@@ -4024,7 +4140,7 @@
       </c>
       <c r="O24" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E24-6,O$5&lt;=$G24),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="P24" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E24-6,P$5&lt;=$G24),"■","")</f>
@@ -4046,19 +4162,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E24-6,T$5&lt;=$G24),"■","")</f>
         <v/>
       </c>
+      <c r="U24" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E24-6,U$5&lt;=$G24),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="14" t="s">
-        <v>189</v>
+        <v>207</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>190</v>
+        <v>208</v>
       </c>
       <c r="C25" s="14" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="E25" s="22" t="n">
         <v>46335</v>
@@ -4071,11 +4191,10 @@
         <v>46346</v>
       </c>
       <c r="H25" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="I25" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E25-6,I$5&lt;=$G25),"■","")</f>
-        <v/>
+        <v>204</v>
+      </c>
+      <c r="I25" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J25" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E25-6,J$5&lt;=$G25),"■","")</f>
@@ -4095,7 +4214,7 @@
       </c>
       <c r="N25" s="25" t="str">
         <f aca="false">IF(AND(N$5&gt;=$E25-6,N$5&lt;=$G25),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="O25" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E25-6,O$5&lt;=$G25),"■","")</f>
@@ -4103,7 +4222,7 @@
       </c>
       <c r="P25" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E25-6,P$5&lt;=$G25),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="Q25" s="25" t="str">
         <f aca="false">IF(AND(Q$5&gt;=$E25-6,Q$5&lt;=$G25),"■","")</f>
@@ -4121,19 +4240,23 @@
         <f aca="false">IF(AND(T$5&gt;=$E25-6,T$5&lt;=$G25),"■","")</f>
         <v/>
       </c>
+      <c r="U25" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E25-6,U$5&lt;=$G25),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="14" t="s">
-        <v>191</v>
+        <v>210</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>192</v>
+        <v>211</v>
       </c>
       <c r="C26" s="14" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="E26" s="22" t="n">
         <v>46335</v>
@@ -4146,11 +4269,10 @@
         <v>46346</v>
       </c>
       <c r="H26" s="14" t="s">
-        <v>183</v>
-      </c>
-      <c r="I26" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E26-6,I$5&lt;=$G26),"■","")</f>
-        <v/>
+        <v>204</v>
+      </c>
+      <c r="I26" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J26" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E26-6,J$5&lt;=$G26),"■","")</f>
@@ -4170,7 +4292,7 @@
       </c>
       <c r="N26" s="25" t="str">
         <f aca="false">IF(AND(N$5&gt;=$E26-6,N$5&lt;=$G26),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="O26" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E26-6,O$5&lt;=$G26),"■","")</f>
@@ -4178,7 +4300,7 @@
       </c>
       <c r="P26" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E26-6,P$5&lt;=$G26),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="Q26" s="25" t="str">
         <f aca="false">IF(AND(Q$5&gt;=$E26-6,Q$5&lt;=$G26),"■","")</f>
@@ -4196,36 +4318,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E26-6,T$5&lt;=$G26),"■","")</f>
         <v/>
       </c>
+      <c r="U26" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E26-6,U$5&lt;=$G26),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="14" t="s">
-        <v>193</v>
+        <v>212</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>194</v>
+        <v>213</v>
       </c>
       <c r="C27" s="14" t="s">
-        <v>70</v>
+        <v>82</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="E27" s="22" t="n">
-        <v>46349</v>
+        <v>46335</v>
       </c>
       <c r="F27" s="23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G27" s="24" t="n">
         <f aca="false">E27+F27*7-3</f>
-        <v>46353</v>
+        <v>46346</v>
       </c>
       <c r="H27" s="14" t="s">
-        <v>196</v>
-      </c>
-      <c r="I27" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E27-6,I$5&lt;=$G27),"■","")</f>
-        <v/>
+        <v>204</v>
+      </c>
+      <c r="I27" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J27" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E27-6,J$5&lt;=$G27),"■","")</f>
@@ -4249,7 +4374,7 @@
       </c>
       <c r="O27" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E27-6,O$5&lt;=$G27),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="P27" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E27-6,P$5&lt;=$G27),"■","")</f>
@@ -4271,36 +4396,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E27-6,T$5&lt;=$G27),"■","")</f>
         <v/>
       </c>
+      <c r="U27" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E27-6,U$5&lt;=$G27),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="14" t="s">
-        <v>197</v>
+        <v>214</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>198</v>
+        <v>215</v>
       </c>
       <c r="C28" s="14" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>188</v>
+        <v>216</v>
       </c>
       <c r="E28" s="22" t="n">
-        <v>46356</v>
+        <v>46349</v>
       </c>
       <c r="F28" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G28" s="24" t="n">
         <f aca="false">E28+F28*7-3</f>
-        <v>46360</v>
+        <v>46353</v>
       </c>
       <c r="H28" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="I28" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E28-6,I$5&lt;=$G28),"■","")</f>
-        <v/>
+        <v>217</v>
+      </c>
+      <c r="I28" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J28" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E28-6,J$5&lt;=$G28),"■","")</f>
@@ -4346,36 +4474,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E28-6,T$5&lt;=$G28),"■","")</f>
         <v/>
       </c>
+      <c r="U28" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E28-6,U$5&lt;=$G28),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="14" t="s">
-        <v>199</v>
+        <v>218</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>200</v>
+        <v>219</v>
       </c>
       <c r="C29" s="14" t="s">
-        <v>58</v>
+        <v>94</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>188</v>
+        <v>209</v>
       </c>
       <c r="E29" s="22" t="n">
-        <v>46363</v>
+        <v>46356</v>
       </c>
       <c r="F29" s="23" t="n">
         <v>1</v>
       </c>
       <c r="G29" s="24" t="n">
         <f aca="false">E29+F29*7-3</f>
-        <v>46367</v>
+        <v>46360</v>
       </c>
       <c r="H29" s="14" t="s">
-        <v>197</v>
-      </c>
-      <c r="I29" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E29-6,I$5&lt;=$G29),"■","")</f>
-        <v/>
+        <v>214</v>
+      </c>
+      <c r="I29" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J29" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E29-6,J$5&lt;=$G29),"■","")</f>
@@ -4421,36 +4552,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E29-6,T$5&lt;=$G29),"■","")</f>
         <v/>
       </c>
+      <c r="U29" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E29-6,U$5&lt;=$G29),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="14" t="s">
-        <v>201</v>
+        <v>220</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>202</v>
+        <v>221</v>
       </c>
       <c r="C30" s="14" t="s">
-        <v>46</v>
+        <v>68</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>195</v>
+        <v>209</v>
       </c>
       <c r="E30" s="22" t="n">
-        <v>46321</v>
+        <v>46363</v>
       </c>
       <c r="F30" s="23" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="G30" s="24" t="n">
         <f aca="false">E30+F30*7-3</f>
-        <v>46374</v>
+        <v>46367</v>
       </c>
       <c r="H30" s="14" t="s">
-        <v>152</v>
-      </c>
-      <c r="I30" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E30-6,I$5&lt;=$G30),"■","")</f>
-        <v/>
+        <v>218</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J30" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E30-6,J$5&lt;=$G30),"■","")</f>
@@ -4462,31 +4596,31 @@
       </c>
       <c r="L30" s="25" t="str">
         <f aca="false">IF(AND(L$5&gt;=$E30-6,L$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="M30" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E30-6,M$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="N30" s="25" t="str">
         <f aca="false">IF(AND(N$5&gt;=$E30-6,N$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="O30" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E30-6,O$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="P30" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E30-6,P$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="Q30" s="25" t="str">
         <f aca="false">IF(AND(Q$5&gt;=$E30-6,Q$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="R30" s="25" t="str">
         <f aca="false">IF(AND(R$5&gt;=$E30-6,R$5&lt;=$G30),"■","")</f>
-        <v>■</v>
+        <v/>
       </c>
       <c r="S30" s="25" t="str">
         <f aca="false">IF(AND(S$5&gt;=$E30-6,S$5&lt;=$G30),"■","")</f>
@@ -4496,36 +4630,39 @@
         <f aca="false">IF(AND(T$5&gt;=$E30-6,T$5&lt;=$G30),"■","")</f>
         <v/>
       </c>
+      <c r="U30" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E30-6,U$5&lt;=$G30),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="14" t="s">
-        <v>203</v>
+        <v>222</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>204</v>
+        <v>223</v>
       </c>
       <c r="C31" s="14" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>205</v>
+        <v>216</v>
       </c>
       <c r="E31" s="22" t="n">
-        <v>46377</v>
+        <v>46321</v>
       </c>
       <c r="F31" s="23" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="G31" s="24" t="n">
         <f aca="false">E31+F31*7-3</f>
-        <v>46381</v>
+        <v>46374</v>
       </c>
       <c r="H31" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="I31" s="25" t="str">
-        <f aca="false">IF(AND(I$5&gt;=$E31-6,I$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>168</v>
+      </c>
+      <c r="I31" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J31" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E31-6,J$5&lt;=$G31),"■","")</f>
@@ -4541,169 +4678,176 @@
       </c>
       <c r="M31" s="25" t="str">
         <f aca="false">IF(AND(M$5&gt;=$E31-6,M$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="N31" s="25" t="str">
         <f aca="false">IF(AND(N$5&gt;=$E31-6,N$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="O31" s="25" t="str">
         <f aca="false">IF(AND(O$5&gt;=$E31-6,O$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="P31" s="25" t="str">
         <f aca="false">IF(AND(P$5&gt;=$E31-6,P$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="Q31" s="25" t="str">
         <f aca="false">IF(AND(Q$5&gt;=$E31-6,Q$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="R31" s="25" t="str">
         <f aca="false">IF(AND(R$5&gt;=$E31-6,R$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="S31" s="25" t="str">
         <f aca="false">IF(AND(S$5&gt;=$E31-6,S$5&lt;=$G31),"■","")</f>
-        <v/>
+        <v>■</v>
       </c>
       <c r="T31" s="25" t="str">
         <f aca="false">IF(AND(T$5&gt;=$E31-6,T$5&lt;=$G31),"■","")</f>
         <v>■</v>
       </c>
+      <c r="U31" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E31-6,U$5&lt;=$G31),"■","")</f>
+        <v/>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="s">
-        <v>206</v>
-      </c>
-      <c r="B32" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="C32" s="21"/>
-      <c r="D32" s="21" t="s">
-        <v>207</v>
-      </c>
-      <c r="E32" s="21"/>
-      <c r="F32" s="21"/>
-      <c r="G32" s="21"/>
-      <c r="H32" s="21"/>
-      <c r="I32" s="21"/>
-      <c r="J32" s="21"/>
-      <c r="K32" s="21"/>
-      <c r="L32" s="21"/>
-      <c r="M32" s="21"/>
-      <c r="N32" s="21"/>
-      <c r="O32" s="21"/>
-      <c r="P32" s="21"/>
-      <c r="Q32" s="21"/>
-      <c r="R32" s="21"/>
-      <c r="S32" s="21"/>
-      <c r="T32" s="21"/>
+      <c r="A32" s="14" t="s">
+        <v>224</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>225</v>
+      </c>
+      <c r="C32" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>226</v>
+      </c>
+      <c r="E32" s="22" t="n">
+        <v>46377</v>
+      </c>
+      <c r="F32" s="23" t="n">
+        <v>1</v>
+      </c>
+      <c r="G32" s="24" t="n">
+        <f aca="false">E32+F32*7-3</f>
+        <v>46381</v>
+      </c>
+      <c r="H32" s="14" t="s">
+        <v>220</v>
+      </c>
+      <c r="I32" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="J32" s="25" t="str">
+        <f aca="false">IF(AND(J$5&gt;=$E32-6,J$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="K32" s="25" t="str">
+        <f aca="false">IF(AND(K$5&gt;=$E32-6,K$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="L32" s="25" t="str">
+        <f aca="false">IF(AND(L$5&gt;=$E32-6,L$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="M32" s="25" t="str">
+        <f aca="false">IF(AND(M$5&gt;=$E32-6,M$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="N32" s="25" t="str">
+        <f aca="false">IF(AND(N$5&gt;=$E32-6,N$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="O32" s="25" t="str">
+        <f aca="false">IF(AND(O$5&gt;=$E32-6,O$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="P32" s="25" t="str">
+        <f aca="false">IF(AND(P$5&gt;=$E32-6,P$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="Q32" s="25" t="str">
+        <f aca="false">IF(AND(Q$5&gt;=$E32-6,Q$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="R32" s="25" t="str">
+        <f aca="false">IF(AND(R$5&gt;=$E32-6,R$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="S32" s="25" t="str">
+        <f aca="false">IF(AND(S$5&gt;=$E32-6,S$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="T32" s="25" t="str">
+        <f aca="false">IF(AND(T$5&gt;=$E32-6,T$5&lt;=$G32),"■","")</f>
+        <v/>
+      </c>
+      <c r="U32" s="25" t="str">
+        <f aca="false">IF(AND(U$5&gt;=$E32-6,U$5&lt;=$G32),"■","")</f>
+        <v>■</v>
+      </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="14" t="s">
-        <v>208</v>
-      </c>
-      <c r="B33" s="4" t="s">
-        <v>209</v>
-      </c>
-      <c r="C33" s="14" t="s">
-        <v>210</v>
-      </c>
-      <c r="D33" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="E33" s="22" t="n">
-        <v>46311</v>
-      </c>
-      <c r="F33" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="G33" s="24" t="n">
-        <f aca="false">E33</f>
-        <v>46311</v>
-      </c>
-      <c r="H33" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="I33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=I$5,$E33&lt;I$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="J33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=J$5,$E33&lt;J$5+7),"◆","")</f>
-        <v>◆</v>
-      </c>
-      <c r="K33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=K$5,$E33&lt;K$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="L33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=L$5,$E33&lt;L$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="M33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=M$5,$E33&lt;M$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="N33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=N$5,$E33&lt;N$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="O33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=O$5,$E33&lt;O$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="P33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=P$5,$E33&lt;P$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="Q33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=Q$5,$E33&lt;Q$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="R33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=R$5,$E33&lt;R$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="S33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=S$5,$E33&lt;S$5+7),"◆","")</f>
-        <v/>
-      </c>
-      <c r="T33" s="25" t="str">
-        <f aca="false">IF(AND($E33&gt;=T$5,$E33&lt;T$5+7),"◆","")</f>
-        <v/>
-      </c>
+      <c r="A33" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="B33" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="C33" s="21"/>
+      <c r="D33" s="21" t="s">
+        <v>228</v>
+      </c>
+      <c r="E33" s="21"/>
+      <c r="F33" s="21"/>
+      <c r="G33" s="21"/>
+      <c r="H33" s="21"/>
+      <c r="I33" s="21"/>
+      <c r="J33" s="21"/>
+      <c r="K33" s="21"/>
+      <c r="L33" s="21"/>
+      <c r="M33" s="21"/>
+      <c r="N33" s="21"/>
+      <c r="O33" s="21"/>
+      <c r="P33" s="21"/>
+      <c r="Q33" s="21"/>
+      <c r="R33" s="21"/>
+      <c r="S33" s="21"/>
+      <c r="T33" s="21"/>
+      <c r="U33" s="21"/>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="14" t="s">
-        <v>212</v>
+        <v>229</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>213</v>
+        <v>230</v>
       </c>
       <c r="C34" s="14" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="E34" s="22" t="n">
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="F34" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G34" s="24" t="n">
         <f aca="false">E34</f>
-        <v>46316</v>
+        <v>46311</v>
       </c>
       <c r="H34" s="14" t="s">
-        <v>176</v>
-      </c>
-      <c r="I34" s="25" t="str">
-        <f aca="false">IF(AND($E34&gt;=I$5,$E34&lt;I$5+7),"◆","")</f>
-        <v/>
+        <v>187</v>
+      </c>
+      <c r="I34" s="14" t="s">
+        <v>233</v>
       </c>
       <c r="J34" s="25" t="str">
         <f aca="false">IF(AND($E34&gt;=J$5,$E34&lt;J$5+7),"◆","")</f>
@@ -4749,36 +4893,39 @@
         <f aca="false">IF(AND($E34&gt;=T$5,$E34&lt;T$5+7),"◆","")</f>
         <v/>
       </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="U34" s="25" t="str">
+        <f aca="false">IF(AND($E34&gt;=U$5,$E34&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="14" t="s">
-        <v>214</v>
+        <v>234</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>215</v>
+        <v>235</v>
       </c>
       <c r="C35" s="14" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="E35" s="22" t="n">
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="F35" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G35" s="24" t="n">
         <f aca="false">E35</f>
-        <v>46325</v>
+        <v>46315</v>
       </c>
       <c r="H35" s="14" t="s">
-        <v>181</v>
-      </c>
-      <c r="I35" s="25" t="str">
-        <f aca="false">IF(AND($E35&gt;=I$5,$E35&lt;I$5+7),"◆","")</f>
-        <v/>
+        <v>195</v>
+      </c>
+      <c r="I35" s="14" t="s">
+        <v>233</v>
       </c>
       <c r="J35" s="25" t="str">
         <f aca="false">IF(AND($E35&gt;=J$5,$E35&lt;J$5+7),"◆","")</f>
@@ -4824,36 +4971,39 @@
         <f aca="false">IF(AND($E35&gt;=T$5,$E35&lt;T$5+7),"◆","")</f>
         <v/>
       </c>
+      <c r="U35" s="25" t="str">
+        <f aca="false">IF(AND($E35&gt;=U$5,$E35&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="14" t="s">
-        <v>216</v>
+        <v>236</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>217</v>
+        <v>237</v>
       </c>
       <c r="C36" s="14" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="E36" s="22" t="n">
-        <v>46353</v>
+        <v>46316</v>
       </c>
       <c r="F36" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G36" s="24" t="n">
         <f aca="false">E36</f>
-        <v>46353</v>
+        <v>46316</v>
       </c>
       <c r="H36" s="14" t="s">
-        <v>193</v>
-      </c>
-      <c r="I36" s="25" t="str">
-        <f aca="false">IF(AND($E36&gt;=I$5,$E36&lt;I$5+7),"◆","")</f>
-        <v/>
+        <v>194</v>
+      </c>
+      <c r="I36" s="14" t="s">
+        <v>238</v>
       </c>
       <c r="J36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=J$5,$E36&lt;J$5+7),"◆","")</f>
@@ -4865,7 +5015,7 @@
       </c>
       <c r="L36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=L$5,$E36&lt;L$5+7),"◆","")</f>
-        <v/>
+        <v>◆</v>
       </c>
       <c r="M36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=M$5,$E36&lt;M$5+7),"◆","")</f>
@@ -4881,7 +5031,7 @@
       </c>
       <c r="P36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=P$5,$E36&lt;P$5+7),"◆","")</f>
-        <v>◆</v>
+        <v/>
       </c>
       <c r="Q36" s="25" t="str">
         <f aca="false">IF(AND($E36&gt;=Q$5,$E36&lt;Q$5+7),"◆","")</f>
@@ -4899,36 +5049,39 @@
         <f aca="false">IF(AND($E36&gt;=T$5,$E36&lt;T$5+7),"◆","")</f>
         <v/>
       </c>
+      <c r="U36" s="25" t="str">
+        <f aca="false">IF(AND($E36&gt;=U$5,$E36&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="14" t="s">
-        <v>218</v>
+        <v>239</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="C37" s="14" t="s">
-        <v>210</v>
+        <v>231</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>211</v>
+        <v>232</v>
       </c>
       <c r="E37" s="22" t="n">
-        <v>46370</v>
+        <v>46325</v>
       </c>
       <c r="F37" s="23" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="24" t="n">
         <f aca="false">E37</f>
-        <v>46370</v>
+        <v>46325</v>
       </c>
       <c r="H37" s="14" t="s">
-        <v>199</v>
-      </c>
-      <c r="I37" s="25" t="str">
-        <f aca="false">IF(AND($E37&gt;=I$5,$E37&lt;I$5+7),"◆","")</f>
-        <v/>
+        <v>201</v>
+      </c>
+      <c r="I37" s="14" t="s">
+        <v>203</v>
       </c>
       <c r="J37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=J$5,$E37&lt;J$5+7),"◆","")</f>
@@ -4944,7 +5097,7 @@
       </c>
       <c r="M37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=M$5,$E37&lt;M$5+7),"◆","")</f>
-        <v/>
+        <v>◆</v>
       </c>
       <c r="N37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=N$5,$E37&lt;N$5+7),"◆","")</f>
@@ -4968,117 +5121,321 @@
       </c>
       <c r="S37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=S$5,$E37&lt;S$5+7),"◆","")</f>
-        <v>◆</v>
+        <v/>
       </c>
       <c r="T37" s="25" t="str">
         <f aca="false">IF(AND($E37&gt;=T$5,$E37&lt;T$5+7),"◆","")</f>
         <v/>
       </c>
+      <c r="U37" s="25" t="str">
+        <f aca="false">IF(AND($E37&gt;=U$5,$E37&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="14" t="s">
+        <v>241</v>
+      </c>
+      <c r="B38" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="C38" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="D38" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E38" s="22" t="n">
+        <v>46353</v>
+      </c>
+      <c r="F38" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="24" t="n">
+        <f aca="false">E38</f>
+        <v>46353</v>
+      </c>
+      <c r="H38" s="14" t="s">
+        <v>214</v>
+      </c>
+      <c r="I38" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="J38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=J$5,$E38&lt;J$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="K38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=K$5,$E38&lt;K$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="L38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=L$5,$E38&lt;L$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="M38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=M$5,$E38&lt;M$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="N38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=N$5,$E38&lt;N$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="O38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=O$5,$E38&lt;O$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="P38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=P$5,$E38&lt;P$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="Q38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=Q$5,$E38&lt;Q$5+7),"◆","")</f>
+        <v>◆</v>
+      </c>
+      <c r="R38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=R$5,$E38&lt;R$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="S38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=S$5,$E38&lt;S$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="T38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=T$5,$E38&lt;T$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="U38" s="25" t="str">
+        <f aca="false">IF(AND($E38&gt;=U$5,$E38&lt;U$5+7),"◆","")</f>
+        <v/>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B39" s="16" t="s">
+      <c r="A39" s="14" t="s">
+        <v>243</v>
+      </c>
+      <c r="B39" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="C39" s="14" t="s">
+        <v>231</v>
+      </c>
+      <c r="D39" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="E39" s="22" t="n">
+        <v>46370</v>
+      </c>
+      <c r="F39" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="24" t="n">
+        <f aca="false">E39</f>
+        <v>46370</v>
+      </c>
+      <c r="H39" s="14" t="s">
         <v>220</v>
       </c>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B40" s="26" t="s">
-        <v>46</v>
+      <c r="I39" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="J39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=J$5,$E39&lt;J$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="K39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=K$5,$E39&lt;K$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="L39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=L$5,$E39&lt;L$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="M39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=M$5,$E39&lt;M$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="N39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=N$5,$E39&lt;N$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="O39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=O$5,$E39&lt;O$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="P39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=P$5,$E39&lt;P$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="Q39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=Q$5,$E39&lt;Q$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="R39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=R$5,$E39&lt;R$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="S39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=S$5,$E39&lt;S$5+7),"◆","")</f>
+        <v/>
+      </c>
+      <c r="T39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=T$5,$E39&lt;T$5+7),"◆","")</f>
+        <v>◆</v>
+      </c>
+      <c r="U39" s="25" t="str">
+        <f aca="false">IF(AND($E39&gt;=U$5,$E39&lt;U$5+7),"◆","")</f>
+        <v/>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B41" s="27" t="s">
-        <v>58</v>
+      <c r="B41" s="16" t="s">
+        <v>245</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B42" s="28" t="s">
-        <v>64</v>
+      <c r="B42" s="26" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B43" s="29" t="s">
-        <v>70</v>
+      <c r="B43" s="27" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B44" s="30" t="s">
-        <v>80</v>
+      <c r="B44" s="28" t="s">
+        <v>76</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B45" s="31" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B47" s="32" t="s">
-        <v>221</v>
-      </c>
-      <c r="C47" s="32"/>
-      <c r="D47" s="32"/>
-      <c r="E47" s="32"/>
-      <c r="F47" s="32"/>
-      <c r="G47" s="32"/>
-      <c r="H47" s="32"/>
-      <c r="I47" s="32"/>
-      <c r="J47" s="32"/>
-      <c r="K47" s="32"/>
-      <c r="L47" s="32"/>
-      <c r="M47" s="32"/>
-      <c r="N47" s="32"/>
-      <c r="O47" s="32"/>
-      <c r="P47" s="32"/>
-      <c r="Q47" s="32"/>
-      <c r="R47" s="32"/>
-      <c r="S47" s="32"/>
-      <c r="T47" s="32"/>
-    </row>
-    <row r="48" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B48" s="32" t="s">
-        <v>222</v>
-      </c>
-      <c r="C48" s="32"/>
-      <c r="D48" s="32"/>
-      <c r="E48" s="32"/>
-      <c r="F48" s="32"/>
-      <c r="G48" s="32"/>
-      <c r="H48" s="32"/>
-      <c r="I48" s="32"/>
-      <c r="J48" s="32"/>
-      <c r="K48" s="32"/>
-      <c r="L48" s="32"/>
-      <c r="M48" s="32"/>
-      <c r="N48" s="32"/>
-      <c r="O48" s="32"/>
-      <c r="P48" s="32"/>
-      <c r="Q48" s="32"/>
-      <c r="R48" s="32"/>
-      <c r="S48" s="32"/>
-      <c r="T48" s="32"/>
+      <c r="B45" s="29" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B46" s="30" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B47" s="31" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B49" s="32" t="s">
+        <v>246</v>
+      </c>
+      <c r="C49" s="32"/>
+      <c r="D49" s="32"/>
+      <c r="E49" s="32"/>
+      <c r="F49" s="32"/>
+      <c r="G49" s="32"/>
+      <c r="H49" s="32"/>
+      <c r="I49" s="32"/>
+      <c r="J49" s="32"/>
+      <c r="K49" s="32"/>
+      <c r="L49" s="32"/>
+      <c r="M49" s="32"/>
+      <c r="N49" s="32"/>
+      <c r="O49" s="32"/>
+      <c r="P49" s="32"/>
+      <c r="Q49" s="32"/>
+      <c r="R49" s="32"/>
+      <c r="S49" s="32"/>
+      <c r="T49" s="32"/>
+      <c r="U49" s="32"/>
+    </row>
+    <row r="50" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B50" s="32" t="s">
+        <v>247</v>
+      </c>
+      <c r="C50" s="32"/>
+      <c r="D50" s="32"/>
+      <c r="E50" s="32"/>
+      <c r="F50" s="32"/>
+      <c r="G50" s="32"/>
+      <c r="H50" s="32"/>
+      <c r="I50" s="32"/>
+      <c r="J50" s="32"/>
+      <c r="K50" s="32"/>
+      <c r="L50" s="32"/>
+      <c r="M50" s="32"/>
+      <c r="N50" s="32"/>
+      <c r="O50" s="32"/>
+      <c r="P50" s="32"/>
+      <c r="Q50" s="32"/>
+      <c r="R50" s="32"/>
+      <c r="S50" s="32"/>
+      <c r="T50" s="32"/>
+      <c r="U50" s="32"/>
+    </row>
+    <row r="51" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B51" s="32" t="s">
+        <v>248</v>
+      </c>
+      <c r="C51" s="32"/>
+      <c r="D51" s="32"/>
+      <c r="E51" s="32"/>
+      <c r="F51" s="32"/>
+      <c r="G51" s="32"/>
+      <c r="H51" s="32"/>
+      <c r="I51" s="32"/>
+      <c r="J51" s="32"/>
+      <c r="K51" s="32"/>
+      <c r="L51" s="32"/>
+      <c r="M51" s="32"/>
+      <c r="N51" s="32"/>
+      <c r="O51" s="32"/>
+      <c r="P51" s="32"/>
+      <c r="Q51" s="32"/>
+      <c r="R51" s="32"/>
+      <c r="S51" s="32"/>
+      <c r="T51" s="32"/>
+      <c r="U51" s="32"/>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B47:T47"/>
-    <mergeCell ref="B48:T48"/>
+  <mergeCells count="3">
+    <mergeCell ref="B49:U49"/>
+    <mergeCell ref="B50:U50"/>
+    <mergeCell ref="B51:U51"/>
   </mergeCells>
-  <conditionalFormatting sqref="I6:T37">
+  <conditionalFormatting sqref="J6:U39">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
-      <formula>AND(I6&lt;&gt;"",$C6="Abraham")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,7)="Abraham")</formula>
     </cfRule>
     <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="4">
-      <formula>AND(I6&lt;&gt;"",$C6="Sebastián")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,9)="Sebastián")</formula>
     </cfRule>
     <cfRule type="expression" priority="4" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="5">
-      <formula>AND(I6&lt;&gt;"",$C6="Lisandra")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,8)="Lisandra")</formula>
     </cfRule>
     <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="6">
-      <formula>AND(I6&lt;&gt;"",$C6="Felipe")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,6)="Felipe")</formula>
     </cfRule>
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="7">
-      <formula>AND(I6&lt;&gt;"",$C6="Bárbara")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,7)="Bárbara")</formula>
     </cfRule>
     <cfRule type="expression" priority="7" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="8">
-      <formula>AND(I6&lt;&gt;"",$C6="Equipo")</formula>
+      <formula>AND(J6&lt;&gt;"",LEFT($C6,6)="Equipo")</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I6:I39">
+    <cfRule type="expression" priority="8" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>I6="Listo"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="9" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+      <formula>I6="Cumplido"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="10" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>I6="En curso"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="11" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+      <formula>I6="Hoy"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="12" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
+      <formula>I6="Pendiente"</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>

</xml_diff>

<commit_message>
docs: dashboard conectado a Cognito (21/10) y mensaje de error con el detalle de Cognito
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015SVKuYduNdeGeu8Q4SMcKp
</commit_message>
<xml_diff>
--- a/docs/nota-2/Induplac_Roles_Equipo.xlsx
+++ b/docs/nota-2/Induplac_Roles_Equipo.xlsx
@@ -1815,8 +1815,10 @@
       <c r="C9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>64</v>
+      <c r="D9" s="4" t="inlineStr">
+        <is>
+          <t>Listo (PR #20, probado el 21/10)</t>
+        </is>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3674,8 +3676,10 @@
       <c r="A18" s="14" t="s">
         <v>189</v>
       </c>
-      <c r="B18" s="4" t="s">
-        <v>190</v>
+      <c r="B18" s="4" t="inlineStr">
+        <is>
+          <t>Cognito con MFA y login del dashboard</t>
+        </is>
       </c>
       <c r="C18" s="14" t="s">
         <v>180</v>
@@ -3696,8 +3700,10 @@
       <c r="H18" s="14" t="s">
         <v>191</v>
       </c>
-      <c r="I18" s="14" t="s">
-        <v>54</v>
+      <c r="I18" s="14" t="inlineStr">
+        <is>
+          <t>Listo</t>
+        </is>
       </c>
       <c r="J18" s="25" t="str">
         <f aca="false">IF(AND(J$5&gt;=$E18-6,J$5&lt;=$G18),"■","")</f>

</xml_diff>